<commit_message>
working on mid-sem tt
</commit_message>
<xml_diff>
--- a/src/outputs/Mid-Sem TT-cleaned.xlsx
+++ b/src/outputs/Mid-Sem TT-cleaned.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CFE8ACD-4840-46AD-9EF5-1C3228733447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B09F45B6-89A3-40FC-8C3B-5C0799C20F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="480">
   <si>
     <t xml:space="preserve">MATH 351%NUMERICAL ANALYSIS%Azure Isaac%ED3-ME%230%Computer Based %Monday, 23 February 2026%Session, 1 (8:15AM - 9:15 AM)%Computer Based </t>
   </si>
@@ -95,43 +95,43 @@
     <t>CE 271%ENGINEERING REPORTING%Tuffour Yaw Adubofour%ED2-CE%260%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2/NAF1%Monday, 23 February 2026%Session, 1 (8:15AM - 9:15 AM)%85/85/50/30/10</t>
   </si>
   <si>
-    <t>EE 467%POWER SYSTEMS OPERATION AND CONTROL%Antoh Emmanuel Kwaku%ED4-EE%224%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%80/80/50/14</t>
-  </si>
-  <si>
-    <t>COE 457%ARTIFICIAL INTELLIGENCE%Nunoo-Mensah Henry%ED4-COE%170%PB201/PB214/PB208/PB212/PB008%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%43/43/30/24/30</t>
-  </si>
-  <si>
-    <t>CHE 255%FLUID TRANSPORT%Momade Zsuzsanna Gál%ED2-CHE%154%NAF1/EA/A110/VCR/ECR%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%45/30/30/25/24</t>
-  </si>
-  <si>
-    <t>CHE 255%FLUID TRANSPORT%Dogbe Eunice Sefakor Aku%ED2-PCE%59%PB014/PB008%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%35/24</t>
-  </si>
-  <si>
-    <t>CE 457%DRAINAGE SYSTEMS%Adjei Kwaku Amaning%ED4-CE%245%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%80/80/55/30</t>
-  </si>
-  <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Dzebre Denis Edem Kwame%ED2-MARI%37%PB014%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%37</t>
-  </si>
-  <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Dzebre Denis Edem Kwame%ED2-AUTO%77%VSLA/LT%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%49/28</t>
-  </si>
-  <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Dzebre Denis Edem Kwame%ED2-IND%80%303/304/206/RMA%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%30/20/20/10</t>
-  </si>
-  <si>
-    <t>BME 471%BIOINSTRUMENTATION II%Acquah Isaac%ED4-BME%84%PB001/PB020%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%42/42</t>
-  </si>
-  <si>
-    <t>MSE 353%PYROMETALLURGY%Agyemang Frank Ofori%ED3-METE%83%VSLA/LT/RMA%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%45/20/18</t>
-  </si>
-  <si>
-    <t>MSE 353%PYROMETALLURGY%Agyemang Frank Ofori%ED3-MSE%89%PB001/PB020%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%45/44</t>
-  </si>
-  <si>
-    <t>PCE 351%SEPARATION PROCESSES I%Dogbe Eunice Sefakor Aku%ED3-PCE%51%N1/N2/206%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%20/20/11</t>
-  </si>
-  <si>
-    <t>TE 451%FUNDAMENTALS OF NETWORK SECURITY%Agyemang Justice Owusu%ED4-TEL%142%PB201/PB214/PB208/PB212%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%44/44/30/24</t>
+    <t>EE 467%POWER SYSTEMS OPERATION AND CONTROL%Antoh Emmanuel Kwaku%ED4-EE%224%VSLA/LT/303/304/206/RMA/RMB/N1/N2%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%45/30/30/20/20/20/20/20/20</t>
+  </si>
+  <si>
+    <t>COE 457%ARTIFICIAL INTELLIGENCE%Nunoo-Mensah Henry%ED4-COE%170%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%85/55/30</t>
+  </si>
+  <si>
+    <t>CHE 255%FLUID TRANSPORT%Momade Zsuzsanna Gál%ED2-CHE%154%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%80/46/28</t>
+  </si>
+  <si>
+    <t>CE 457%DRAINAGE SYSTEMS%Adjei Kwaku Amaning%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB212%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%45/45/45/45/45/20</t>
+  </si>
+  <si>
+    <t>ME 255%STRENGTH OF MATERIALS I%Dzebre Denis Edem Kwame%ED2-MARI%37%N1/N2%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%20/17</t>
+  </si>
+  <si>
+    <t>ME 255%STRENGTH OF MATERIALS I%Dzebre Denis Edem Kwame%ED2-AUTO%77%EA/ECR/VCR%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%30/25/22</t>
+  </si>
+  <si>
+    <t>ME 255%STRENGTH OF MATERIALS I%Dzebre Denis Edem Kwame%ED2-IND%80%303/304/206/RMB%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%22/20/20/18</t>
+  </si>
+  <si>
+    <t>BME 471%BIOINSTRUMENTATION II%Acquah Isaac%ED4-BME%84%PB008/PB208/PB212%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%30/30/24</t>
+  </si>
+  <si>
+    <t>MSE 353%PYROMETALLURGY%Agyemang Frank Ofori%ED3-METE%83%VSLA/LT/RMA%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%40/25/18</t>
+  </si>
+  <si>
+    <t>MSE 353%PYROMETALLURGY%Agyemang Frank Ofori%ED3-MSE%89%NAF1/A110/VCR%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%40/30/19</t>
+  </si>
+  <si>
+    <t>PCE 351%SEPARATION PROCESSES I%Dogbe Eunice Sefakor Aku%ED3-PCE%51%NEB-GF%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%51</t>
+  </si>
+  <si>
+    <t>EE 265%ELECTRICAL SERVICES DESIGN%Kwegyir Daniel%ED2-EE%340%PB001/PB020/PB014/PB201/PB214/PB008/PB208/NEB-GF%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%PB001/PB020/PB014/PB201/PB214/PB008/PB208/NEB-GF</t>
+  </si>
+  <si>
+    <t>TE 451%FUNDAMENTALS OF NETWORK SECURITY%Agyemang Justice Owusu%ED4-TEL%142%NEB-TF%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%142</t>
   </si>
   <si>
     <t>AE 453%ENVIRONMENTAL CONTROL AND LIVESTOCK HOUSING%Lavie Jerome Dela%ED4-AE%103%NAF1/EA/A110/ECR%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%40/25/25/13</t>
@@ -188,12 +188,6 @@
     <t>ME 473%COMPUTER AIDED DESIGN AND MANUFACTURING%Afriyie Nyarko Frank Kwabena%ED4-ME%144%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 3 (11:45AM - 12:45 PM)%80/50/14</t>
   </si>
   <si>
-    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-ME%242%PB001/PB020/PB014/PB201/PB214/PB212%Monday, 23 February 2026%Session, 3 (11:45AM - 12:45 PM)%45/45/45/45/45/17</t>
-  </si>
-  <si>
-    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-AERO%74%N1/N2/206%Monday, 23 February 2026%Session, 3 (11:45AM - 12:45 PM)%25/25/24</t>
-  </si>
-  <si>
     <t>ME 159%TECHNICAL DRAWING%Oppong Tawiah Peter%ED1-PE%129%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 3 (11:45AM - 12:45 PM)%70/30/29</t>
   </si>
   <si>
@@ -206,10 +200,10 @@
     <t>ME 265%THERMODYNAMICS I%Forson Francis Kofi%ED2-AE%155%PB001/PB020/PB014/PB212%Monday, 23 February 2026%Session, 3 (11:45AM - 12:45 PM)%45/45/45/20</t>
   </si>
   <si>
-    <t>METE 457%CORROSION OF ENGINEERING MATERIALS%Arthur Emmanuel Kwesi%ED4-METE%49%VSLA%Monday, 23 February 2026%Session, 3 (11:45AM - 12:45 PM)%49</t>
-  </si>
-  <si>
-    <t>MSE 453%CORROSION OF ENGINEERING MATERIALS%Arthur Emmanuel Kwesi%ED4-MSE%64%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 3 (11:45AM - 12:45 PM)%20/30/22</t>
+    <t>METE 457%CORROSION OF ENGINEERING MATERIALS%Andrews Anthony%ED4-METE%49%VSLA%Monday, 23 February 2026%Session, 3 (11:45AM - 12:45 PM)%49</t>
+  </si>
+  <si>
+    <t>MSE 453%CORROSION OF ENGINEERING MATERIALS%Andrews Anthony%ED4-MSE%64%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 3 (11:45AM - 12:45 PM)%20/30/22</t>
   </si>
   <si>
     <t>ENGL 157%COMMUNICATION SKILLS I%Sarfo-Adu Kwasi%ED1-CHE%120%Computer Based%Monday, 23 February 2026%Session, 4 (1:30PM - 2:30 PM)%120</t>
@@ -287,49 +281,43 @@
     <t>ENGL 157%COMMUNICATION SKILLS I%Alhassan Yakubu%ED1-METE%72%Computer Based%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%72</t>
   </si>
   <si>
-    <t>COE 261%COMMUNICATION SYSTEMS%Tchao Eric Tutu%ED2-COE%253%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%85/85/55/30/28</t>
-  </si>
-  <si>
-    <t>CE 367%TRANSPORTATION ENGINEERING I%Tutu Kenneth Adomako%ED3-CE%223%PB001/PB020/PB014/PB201/PB214%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%45/45/45/45/43</t>
-  </si>
-  <si>
-    <t>PCE 359%PETROLEUM FLUID PROPERTIES%Adenutsi Caspar Daniel%ED3-PCE%51%PB208/PB212%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%30/21</t>
-  </si>
-  <si>
-    <t>GED 251%MINERALOGY%Wilson Matthew Coffie%ED2-METE%59%N1/N2/RMA%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%20/20/19</t>
-  </si>
-  <si>
-    <t>GED 251%MINERALOGY%Wilson Matthew Coffie%ED2-GEOL%154%VSLA/LT/303/206/304%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%50/30/30/24/20</t>
-  </si>
-  <si>
-    <t>IE 351%OPERATIONS RESEARCH I%Mensah Lena Dzifa%ED3-IND%72%PB214/PB008 %Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%42/30</t>
-  </si>
-  <si>
-    <t>TE 255%INTRODUCTION TO PROGRAMMING II%Agyemang Justice Owusu%ED2-TEL%179%PB001/PB020/PB014/PB201%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%45/45/45/44</t>
-  </si>
-  <si>
-    <t>GED 375%PRINCIPLES OF ENGINEERING GEOLOGY%Gidigasu Solomon Senyo Robert%ED3-GEOL%154%VSLA/LT/303/206/304%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%50/30/30/20/24</t>
-  </si>
-  <si>
-    <t>MME 467%MARINE INTERNAL COMBUSTION ENGINES%Amoabeng Kofi Owura%ED4-MARI%23%VCR %Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%23</t>
-  </si>
-  <si>
-    <t>AE 459%ADVANCED FARM POWER AND MACHINERY%Aikins Stephen Hill Mends%ED4-AE%103%NAF1/EA/A110%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%43/30/30</t>
-  </si>
-  <si>
-    <t>COE 251%C PROGRAMMING%Adjei Prince Ebenezer%ED2-EE%376%NAF1/NEB-SF/NEB-TF/NEB-FF1/NEB-FF2/EA/A110/VCR%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%45/85/85/55/30/30/30/16</t>
+    <t>COE 261%COMMUNICATION SYSTEMS%Tchao Eric Tutu%ED2-COE%253%PB001/PB020/PB014/PB201/PB214/PB208/PB212%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%40/40/40/40/40/30/23</t>
+  </si>
+  <si>
+    <t>CE 367%TRANSPORTATION ENGINEERING I%Tutu Kenneth Adomako%ED3-CE%223%VSLA/LT/303/304/206/RMA/RMB/N1/N2%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%40/28/28/22/22/22/22/22/17</t>
+  </si>
+  <si>
+    <t>PCE 359%PETROLEUM FLUID PROPERTIES%Adenutsi Caspar Daniel%ED3-PCE%51%EA/A110%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%25/26</t>
+  </si>
+  <si>
+    <t>GED 251%MINERALOGY%Wilson Matthew Coffie%ED2-METE%59%NAF1/VCR%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%40/19</t>
+  </si>
+  <si>
+    <t>IE 351%OPERATIONS RESEARCH I%Mensah Lena Dzifa%ED3-IND%72%VSLA/RMA/RMB%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%40/16/16</t>
+  </si>
+  <si>
+    <t>TE 255%INTRODUCTION TO PROGRAMMING II%Agyemang Justice Owusu%ED2-TEL%179%NEB-TF%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%NEB-TF</t>
+  </si>
+  <si>
+    <t>GED 375%PRINCIPLES OF ENGINEERING GEOLOGY%Gidigasu Solomon Senyo Robert%ED3-GEOL%154%NAF1/A110/EA/VCR/ECR%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%45/30/30/25/25</t>
+  </si>
+  <si>
+    <t>MME 467%MARINE INTERNAL COMBUSTION ENGINES%Amoabeng Kofi Owura%ED4-MARI%23%PB008%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%23</t>
+  </si>
+  <si>
+    <t>AE 459%ADVANCED FARM POWER AND MACHINERY%Aikins Stephen Hill Mends%ED4-AE%103%NEB-SF/NEB-FF2%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%80/23</t>
+  </si>
+  <si>
+    <t>COE 251%C PROGRAMMING%Adjei Prince Ebenezer%ED2-EE%340%PB001/PB020/PB014/PB201/PB214/PB008/PB208/PB212/NEB-FF1%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%45/45/45/45/45/30/30/25/30</t>
   </si>
   <si>
     <t>AE 381%COMPUTER APPLICATION FOR AGRICULTURAL ENGINEERS%Amponsah William%ED3-AE%105%Computer Based%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%105</t>
   </si>
   <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Andoh Prince Yaw%ED2-PE%97%VSLA/LT/RMA%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%50/30/17</t>
-  </si>
-  <si>
     <t>CE 471%IRRIGATION AND DRAINAGE ENGINEERING%Anornu Geophrey Kwame%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB212%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%45/45/45/45/45/20</t>
   </si>
   <si>
-    <t>CHE 471%PHARMACEUTICAL TECHNOLOGY%Johnson Raphael%ED4-PCE%36%206/304%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%20/16</t>
+    <t>CHE 471%PHARMACEUTICAL TECHNOLOGY%Johnson Raphael%ED4-PCE%36%A110/EA%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%20/16</t>
   </si>
   <si>
     <t>ENGL 263%LITERATURE IN ENGLISH I%Yeboah Philomena Ama Okyeso%ED2-AERO%74%303/304/206%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%25/25/24</t>
@@ -350,15 +338,18 @@
     <t>IE 451%FACILITIES DESIGN AND MATERIAL HANDLING%Sackey Samuel Mensah%ED4-IND%67%PB008/PB208/PB212%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%20/20/17</t>
   </si>
   <si>
-    <t>AERO 483%AVIONICS%Oppong David Kofi%ED4-AERO%61%NAF1/A110%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%40/21</t>
-  </si>
-  <si>
-    <t>ME 483%MECHATRONICS%Sackey Samuel Mensah%ED4-ME%144%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%NEB-SF/NEB-FF1/NEB-FF2</t>
+    <t>AERO 483%AVIONICS%Oppong David Kofi%ED4-AERO%61%NEB-TF%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%61</t>
+  </si>
+  <si>
+    <t>ME 483%MECHATRONICS%Sackey Samuel Mensah%ED4-ME%144%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%75/45/24</t>
   </si>
   <si>
     <t>EE 463%SPECIAL ELECTRICAL MACHINES%Kwegyir Daniel%ED4-EE%224%PB001/PB020/PB014/PB201/PB214%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%45/45/45/45/44</t>
   </si>
   <si>
+    <t>CHE 467%BIOCHEMICAL TECHNOLOGY%Ankudey Emmanuel Godwin%ED4-CHE%31%NAF1%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%31</t>
+  </si>
+  <si>
     <t>TE 351%INFORMATION THEORY AND CODING%Obour Agyekum Kwame Opuni-Boachie%ED3-TEL%147%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 6 (5:00PM - 6:00 PM)%80/45/22</t>
   </si>
   <si>
@@ -386,13 +377,13 @@
     <t>COE 363%DATA STRUCTURES AND ALGORITHMS%Adjaidoo Theresa-Samuelle Maame Atwemaah%ED3-COE%276%Computer Based%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%276</t>
   </si>
   <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Barnes Benedict%ED2-EE%376%NAF1/NEB-SF/NEB-TF/NEB-FF1/NEB-FF2/EA/A110/VCR%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/85/85/55/30/30/30/16</t>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Barnes Benedict%ED2-EE%340%NAF1/NEB-SF/NEB-TF/NEB-FF1/NEB-FF2/EA/A110%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/80/80/55/30/30/30/26</t>
   </si>
   <si>
     <t>MATH 251%DIFFERENTIAL EQUATIONS%Barnes Benedict%ED2-CHE%154%VSLA/LT/303/206/304%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%50/30/30/24/20</t>
   </si>
   <si>
-    <t>MSE 357%FOUNDRY TECHNOLOGY%Bota Osei Sekyere%ED3-MSE%89%PB014/PB214%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/44</t>
+    <t>MSE 357%FOUNDRY TECHNOLOGY%Bota Osei Sekyere%ED3-MSE%89%PB214/PB201%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/44</t>
   </si>
   <si>
     <t>MSE 357%FOUNDRY TECHNOLOGY%Bota Osei Sekyere%ED3-METE%83%A110/VCR/ECR%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%30/26/27</t>
@@ -401,25 +392,25 @@
     <t>GED 357%BASIC HYDROLOGY%Appiah-Adjei Emmanuel Kwame%ED3-GEOL%154%VSLA/LT/303/206/304%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%50/30/30/20/24</t>
   </si>
   <si>
-    <t>AE 353%AGRICULTURAL MATERIALS HANDLING AND PROCESSING%Akowuah Joseph Oppong%ED3-AE%105%PB014/PB214/PB212%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/45/15</t>
-  </si>
-  <si>
-    <t>TE 457%EMERGING TRENDS IN COMMUNICATION%Kponyo Jerry John%ED4-TEL%142%NEB-TF/NAF1/EA%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%80/40/22</t>
-  </si>
-  <si>
-    <t>PE 353%DRILLING ENGINEERING I%Adjei Stephen%ED3-PE%82%RMA/RMB/N2/N1%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20/20/22</t>
-  </si>
-  <si>
-    <t>CHE 361%SILICATE TECHNOLOGY I%Momade Zsuzsanna Gál%ED3-CHE%15%PB001/PB020/PB212%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%15</t>
+    <t>AE 353%AGRICULTURAL MATERIALS HANDLING AND PROCESSING%Akowuah Joseph Oppong%ED3-AE%105%PB001/PB020/PB008%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/40/25</t>
+  </si>
+  <si>
+    <t>TE 457%EMERGING TRENDS IN COMMUNICATION%Kponyo Jerry John%ED4-TEL%142%PB001/PB020/PB014/PB212%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/40/40/22</t>
+  </si>
+  <si>
+    <t>PE 353%DRILLING ENGINEERING I%Adjei Stephen%ED3-PE%82%NEB-TF%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20/20/22</t>
+  </si>
+  <si>
+    <t>CHE 361%SILICATE TECHNOLOGY I%Momade Zsuzsanna Gál%ED3-CHE%15%PB212%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%15</t>
   </si>
   <si>
     <t>BME 451%MEDICAL IMAGING II%Kotei Addison Eric Clement%ED4-BME%84%RMA/RMB/N1/N2%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20/24/20</t>
   </si>
   <si>
-    <t>ME 467%RENEWABLE ENERGY CONVERSION%Quansah David Ato%ED4-AERO%61%PB208/PB008%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%30/31</t>
-  </si>
-  <si>
-    <t>PE 465%INSTRUMENTATION AND CONTROL%Sarkodie Kwame%ED4-PE%103%PB001/PB020/PB212%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/45/13</t>
+    <t>ME 467%RENEWABLE ENERGY CONVERSION%Quansah David Ato%ED4-AERO%61%PB014/PB008%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/21</t>
+  </si>
+  <si>
+    <t>PE 465%INSTRUMENTATION AND CONTROL%Sarkodie Kwame%ED4-PE%103%PB201/PB214/PB208%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/40/23</t>
   </si>
   <si>
     <t>ME 477%PRODUCTION ENGINEERING%Obeng George Yaw%ED4-ME%144%NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 1 (8:15 AM - 9:15 AM)%75/45/24</t>
@@ -464,6 +455,9 @@
     <t>MATH 151%ALGEBRA%Barnes Benedict%ED1-CHE%120%VSLA/LT/304/RMA%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%46/25/25/24</t>
   </si>
   <si>
+    <t>MATH 151%ALGEBRA%Barnes Benedict%ED1-PCE%56%PB008/PB208%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/26</t>
+  </si>
+  <si>
     <t>MATH 151%ALGEBRA%Adu-Ansah Lawton%ED1-TEL%129%VSLA/LT/304/RMA%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/30/25/24</t>
   </si>
   <si>
@@ -476,58 +470,52 @@
     <t>MATH 151%ALGEBRA%Azure Isaac%ED1-GEOM%100%RMB/303/N1/N2%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%22/30/24/24</t>
   </si>
   <si>
-    <t>Section, 3 ( 11:45 AM - 12:45 PM)%%%%%%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%Section, 3 ( 11:45 AM - 12:45 PM)</t>
-  </si>
-  <si>
-    <t>CHE 357%EXPERIMENTAL DATA ANALYSIS%Kwao-Boateng Emmanuela%ED3-PCE%51%A110/VCR%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%28/23</t>
-  </si>
-  <si>
-    <t>TE 357%OPTICAL COMMUNICATION%Gadze James Dzisi%ED3-TEL%147%PB020/PB201/PB214/PB212%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/40/40/25</t>
-  </si>
-  <si>
-    <t>IE 355%DISCRETE EVENT SIMULATION%Takyi Gabriel%ED3-IND%72%VSLA/303%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%44/28</t>
-  </si>
-  <si>
-    <t>AE 457%CROP PROCESSING%Darko Joseph Ofei %ED4-AE%103%VSLA/LT/RMA/RMB%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/25/20/18</t>
-  </si>
-  <si>
-    <t>GED 459%EXPLORATION GEOCHEMISTRY%Gawu Simon Kafui Yawo%ED4-GEOL%102%LT/N1/RMA/RMB/N2%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%22/22/20/20/20</t>
-  </si>
-  <si>
-    <t>CE 467%HIGHWAY ENGINEERING II%Tuffour Yaw Adubofour%ED4-CE%245%PB001/PB014/PB201/PB214/PB208/PB008/PB212%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%42/42/42/42/30/28/20</t>
-  </si>
-  <si>
-    <t>COE 485%COMPUTER ARCHITECTURE%Boateng Kwame Osei%ED4-COE%170%PB001/PB014/PB020/PB208/PB008%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/40/40/25/25</t>
-  </si>
-  <si>
-    <t>TE 481%WIRELESS DATA COMMUNICATION NETWORK%Opare Kwasi Adu-Boahen%ED4-EE%224%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%75/75/50/24</t>
-  </si>
-  <si>
-    <t>IE 459%RISK ANALYSIS%Asiedu Charlotte%ED4-IND%67%NAF1/EA%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/27</t>
-  </si>
-  <si>
-    <t>CE 355%HYDROLOGY%Adjei Kwaku Amaning%ED3-CE%223%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%75/75/50/23</t>
-  </si>
-  <si>
-    <t>PCE 455%POLLUTION CONTROL IN PETROCHEMICAL INDUSTRY%Kwao-Boateng Emmanuela%ED4-PCE%62%303/206/304%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%22/20/20</t>
-  </si>
-  <si>
-    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-MARI%23%ECR%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%23</t>
-  </si>
-  <si>
-    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-AUTO%32%N1/N2%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%16/16</t>
-  </si>
-  <si>
-    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-ME%144%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/30/30/20/20</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Boateng Maxwell Akwasi%ED2-MARI%37%PB008/PB212%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%19/18</t>
+    <t>TE 357%OPTICAL COMMUNICATION%Gadze James Dzisi%ED3-TEL%147%PB020/PB201/PB214/PB212%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/40/40/25</t>
+  </si>
+  <si>
+    <t>IE 355%DISCRETE EVENT SIMULATION%Takyi Gabriel%ED3-IND%72%VSLA/303%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%44/28</t>
+  </si>
+  <si>
+    <t>AE 457%CROP PROCESSING%Darko Joseph Ofei %ED4-AE%103%VSLA/LT/RMA/RMB%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/25/20/18</t>
+  </si>
+  <si>
+    <t>GED 459%EXPLORATION GEOCHEMISTRY%Gawu Simon Kafui Yawo%ED4-GEOL%102%LT/N1/RMA/RMB/N2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%22/22/20/20/20</t>
+  </si>
+  <si>
+    <t>CE 467%HIGHWAY ENGINEERING II%Tuffour Yaw Adubofour%ED4-CE%245%PB001/PB014/PB201/PB214/PB208/PB008/PB212%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%42/42/42/42/30/28/20</t>
+  </si>
+  <si>
+    <t>COE 485%COMPUTER ARCHITECTURE%Boateng Kwame Osei%ED4-COE%170%PB001/PB014/PB020/PB208/PB008%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/40/40/25/25</t>
+  </si>
+  <si>
+    <t>TE 481%WIRELESS DATA COMMUNICATION NETWORK%Opare Kwasi Adu-Boahen%ED4-EE%224%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%75/75/50/24</t>
+  </si>
+  <si>
+    <t>IE 459%RISK ANALYSIS%Asiedu Charlotte%ED4-IND%67%NAF1/EA%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/27</t>
+  </si>
+  <si>
+    <t>CE 355%HYDROLOGY%Adjei Kwaku Amaning%ED3-CE%223%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%75/75/50/23</t>
+  </si>
+  <si>
+    <t>PCE 455%POLLUTION CONTROL IN PETROCHEMICAL INDUSTRY%Kwao-Boateng Emmanuela%ED4-PCE%62%303/206/304%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%22/20/20</t>
+  </si>
+  <si>
+    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-MARI%23%ECR%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%23</t>
+  </si>
+  <si>
+    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-AUTO%32%N1/N2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%16/16</t>
+  </si>
+  <si>
+    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-ME%144%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%45/30/30/20/20</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Boateng Maxwell Akwasi%ED2-MARI%37%206/RMB%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%20/17</t>
   </si>
   <si>
     <t>MATH 251%DIFFERENTIAL EQUATIONS%Boateng Maxwell Akwasi%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%80/80/55/27</t>
   </si>
   <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-TEL%179%VSLA/LT/303/N1/N2/RMA/RMB%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/28/28/22/22/20/20</t>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-TEL%179%VSLA/LT/303/N1/N2/RMA%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/30/30/25/24/20</t>
   </si>
   <si>
     <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-GEOL%154%VSLA/303/N1/RMA/RMB/304%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/25/25/20/20/20</t>
@@ -554,6 +542,9 @@
     <t>AERO 473%AEROSPACE VEHICLE DESIGN%Oppong David Kofi%ED4-AERO%61%NAF1/ECR%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/21</t>
   </si>
   <si>
+    <t>CHE 357%EXPERIMENTAL DATA ANALYSIS%Kwao-Boateng Emmanuela%ED3-PCE%51%PB008/PB212%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/21</t>
+  </si>
+  <si>
     <t>CHE 357%EXPERIMENTAL DATA ANALYSIS%Rockson Mizpah Ama Dziedzorm%ED3-CHE%100%LT/206/N2/304%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/25/24/24</t>
   </si>
   <si>
@@ -599,22 +590,22 @@
     <t>GE 463%LAND AND GEOGRAPHIC INFORMATION SYSTEM I%Forkuo Eric Kwabena%ED4-GEOM%93%PB201/PB214/PB212%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/40/13</t>
   </si>
   <si>
-    <t>MME 373%DESIGN OF MARINE MACHINE ELEMENTS%Andoh Prince Yaw%ED3-MARI%40%N1/N2%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20</t>
-  </si>
-  <si>
-    <t>AME 373%DESIGN OF AUTO MECHANICAL SYSTEMS%Andoh Prince Yaw%ED3-AUTO%47%RMA/RMB%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%24/24</t>
-  </si>
-  <si>
-    <t>PCE 253%INTRODUCTION TO PETROCHEMICAL INDUSTRIES%Baidoo Martina Francisca%ED2-PCE%59%206/N1/N2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%24/20/15</t>
-  </si>
-  <si>
-    <t>CHE 259%CHEMICAL PROCESS INDUSTRIES%Afotey Benjamin%ED2-CHE%154%VSLA/LT/303/RMA/RMB/304%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/28/28/20/20/18</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Adam Faisal Wahib%ED1-GEOL%119%NAF1/EA/A110/ECR/VCR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%35/22/22/20/20</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Opoku Richard%ED1-CE%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/80/55/27</t>
+    <t>MME 373%DESIGN OF MARINE MACHINE ELEMENTS%Andoh Prince Yaw%ED3-MARI%40%Computer Based%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40</t>
+  </si>
+  <si>
+    <t>AME 373%DESIGN OF AUTO MECHANICAL SYSTEMS%Andoh Prince Yaw%ED3-AUTO%47%Computer Based%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%47</t>
+  </si>
+  <si>
+    <t>PCE 253%INTRODUCTION TO PETROCHEMICAL INDUSTRIES%Baidoo Martina Francisca%ED2-PCE%59%NEB-TF%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%59</t>
+  </si>
+  <si>
+    <t>CHE 259%CHEMICAL PROCESS INDUSTRIES%Afotey Benjamin%ED2-CHE%154%NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/50/24</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Adam Faisal Wahib%ED1-GEOL%119%NAF1/EA/A110/ECR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/27/27/20</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Opoku Richard%ED1-CE%242%VSLA/LT/303/304/RMA/RMB/206/N1/N2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/30/30/25/24/24/20/20/20</t>
   </si>
   <si>
     <t>CE 367%HIGHWAY AND TRANSPORTATION ENGINEERING I%Ababio-Donkor Augustus%ED3-GEOM%115%VSLA/LT/303/304%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%43/26/26/20</t>
@@ -635,21 +626,15 @@
     <t>TE 463%AVIATION COMMUNICATION%Obeng Kwakye Kingsford Sarkodie%ED4-TEL%142%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/30/30/22/20</t>
   </si>
   <si>
-    <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-PE%3%206%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%3</t>
+    <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-CHE%39%206/VCR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%24/15</t>
+  </si>
+  <si>
+    <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-PE%3%ECR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%3</t>
   </si>
   <si>
     <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-PCE%45%PB208/PB212%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%25/20</t>
   </si>
   <si>
-    <t>CHEM 169%PRACTICAL CHEMISTRY I%Opoku Francis%ED1-CHE%120%VSLA/LT/303/304%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%43/27/27/23</t>
-  </si>
-  <si>
-    <t>CHEM 169%PRACTICAL CHEMISTRY I%Opoku Francis%ED1-PCE%56%EA/A110%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%30/26</t>
-  </si>
-  <si>
-    <t>CHEM 169%PRACTICAL CHEMISTRY I%Opoku Francis%ED1-PE%129%PB201/PB214/PB208/PB212%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/40/28/21</t>
-  </si>
-  <si>
     <t>ME 281%ENGINEERING MATERIALS I%Amoabeng Kofi Owura%ED2-AERO%74%A110/EA/VCR%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%28/28/18</t>
   </si>
   <si>
@@ -686,16 +671,13 @@
     <t>ME 465%AIR CONDITIONING AND REFRIGERATION%Sekyere Charles Kofi Kafui%ED4-ME%144%PB001/PB014/PB020/PB008%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/40/40/25</t>
   </si>
   <si>
-    <t>MME 355%BASIC SHIP STRUCTURE%Andoh Prince Yaw%ED3-MARI%40%RMA/RMB%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20</t>
-  </si>
-  <si>
     <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Darko Jeel Pharis%ED3-CHE%64%303/206/304%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%24/20/20</t>
   </si>
   <si>
     <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED1-CE%136%PB201/PB214/PB208/PB212%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/40/30/26</t>
   </si>
   <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED1-GEOL%80%NEB-TF%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%80</t>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED1-GEOL%80%RMB/N1/N2/304%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%20/20/20/20</t>
   </si>
   <si>
     <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED2-BME%42%NAF1%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%42</t>
@@ -725,7 +707,7 @@
     <t>METE 151%INTRODUCTION TO METALLURGICAL ENGINEERING%Koomson Bennetta%ED1-METE%72%NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%47/25</t>
   </si>
   <si>
-    <t>AERO 157%INTRODUCTION TO AVIATION TECHNOLOGY%Oppong David Kofi%ED1-AERO%70%RMB/N1/N2%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%24/24/22</t>
+    <t>AERO 157%INTRODUCTION TO AVIATION TECHNOLOGY%Oppong David Kofi%ED1-AERO%70%NEB-TF%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%70</t>
   </si>
   <si>
     <t>CHEM 151%GENERAL CHEMISTRY%Sarpong Lilian%ED1-BME%136%NAF1/EA/A110/VCR/ECR%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/28/28/20/20</t>
@@ -806,16 +788,16 @@
     <t>STAT 253%PROBABILITY AND STATISTICS%Okutu John Kwadey%ED3-EE%254%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/40/40/40/40/27/27</t>
   </si>
   <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Adu Alfred Asiwome%ED3-MARI%40%PB212%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Adu Alfred Asiwome%ED3-GEOL%154%NAF1/EA/A110/VCR/ECR%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25/25</t>
+    <t>STAT 253%PROBABILITY AND STATISTICS%David Benteh%ED3-MARI%40%PB212%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%David Benteh%ED3-GEOL%154%NAF1/EA/A110/VCR/ECR%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25/25</t>
   </si>
   <si>
     <t>STAT 253%PROBABILITY AND STATISTICS%Okutu John Kwadey%ED3-AUTO%47%VCR/ECR%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%24/24</t>
   </si>
   <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Adu Alfred Asiwome%ED3-BME%94%NAF1/EA/A110%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/27/27</t>
+    <t>STAT 253%PROBABILITY AND STATISTICS%David Benteh%ED3-BME%94%NAF1/EA/A110%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/27/27</t>
   </si>
   <si>
     <t>STAT 253%PROBABILITY AND STATISTICS%Benteh David%ED3-MSE%89%LT/N2/RMA/RMB%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%25/22/20/20</t>
@@ -827,7 +809,7 @@
     <t>STAT 253%PROBABILITY AND STATISTICS%Awiakye-Marfo George%ED3-CE%223%PB014/PB020/PB201/PB214/PB008/PB208%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%42/42/42/42/28/27</t>
   </si>
   <si>
-    <t>CE 255%THEORY OF STRUCTURES%Owusu Twumasi Jones%ED2-GEOL%154%VSLA/LT/303/RMA/RMB/304%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/25/25/20/20/24</t>
+    <t>CE 255%THEORY OF STRUCTURES%Ampofo James Wiafe%ED2-GEOL%154%VSLA/LT/303/RMA/RMB/304%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/25/25/20/20/24</t>
   </si>
   <si>
     <t>CE 255%THEORY OF STRUCTURES%Ampofo James Wiafe%ED2-CE%260%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2/PB001%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%75/75/50/25/35</t>
@@ -842,10 +824,10 @@
     <t>CHE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-CHE%120%NAF1/EA/A110/VCR%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30/20</t>
   </si>
   <si>
-    <t>CHE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-PCE%56%206/N2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%28/28</t>
-  </si>
-  <si>
-    <t>PE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-PE%129%NAF1/EA/A110/ECR%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/30/30/24</t>
+    <t>CHE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-PCE%56%NEB-FF1%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%56</t>
+  </si>
+  <si>
+    <t>PE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-PE%129%VSLA/LT/303/206/N2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/25/20/14</t>
   </si>
   <si>
     <t>MSE 153%INTRODUCTION TO INFORMATION TECHNOLOGY%Okae James%ED1-MSE%98%304/N1/RMA/RMB%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25/24/24</t>
@@ -860,10 +842,10 @@
     <t>TE 353%RANDOM VARIABLES AND STOCHASTIC PROCESSES%Obour Agyekum Kwame Opuni-Boachie%ED3-TEL%147%PB001/PB020/PB014/PB212%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/12</t>
   </si>
   <si>
-    <t>ME 355%STRENGTH OF MATERIALS II%Agyei Agyemang Anthony%ED3-AE%105%VSLA/LT/303%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%50/30/25</t>
-  </si>
-  <si>
-    <t>AE 471%FARM STRUCTURES%Bart Plange Ato%ED4-AE%103%VSLA/LT/303%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%50/30/23</t>
+    <t>ME 355%STRENGTH OF MATERIALS II%Agyei Agyemang Anthony%ED3-AE%105%NEB-SF/NEB-FF2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%80/23</t>
+  </si>
+  <si>
+    <t>AE 471%FARM STRUCTURES%Bart Plange Ato%ED4-AE%103%NAF1/EA/A110%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%43/30/30</t>
   </si>
   <si>
     <t>GE 451%GEODETIC SURVEYING II%Fosu Collins%ED4-GEOM%93%304/N1/RMA/RMB%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/24/22/22</t>
@@ -872,37 +854,40 @@
     <t>EE 167%OCCUPATIONAL HEALTH AND SAFETY%Asiedu Charlotte%ED1-EE%287%PB001/PB020/PB014/PB201/PB214/PB008/PB208/PB212%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/40/40/26/26/20</t>
   </si>
   <si>
-    <t>PE 367%STATISTICS FOR PETROLEUM ENGINEERS%Adjei Stephen%ED3-PE%82%NEB-TF/NEB-FF2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%60/22</t>
-  </si>
-  <si>
-    <t>BME 463%BIOMATERIALS II%Agyapong Dorothy Araba Yakoba%ED4-BME%84%NEB-TF/NEB-FF2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%65/19</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Oppong Tawiah Peter%ED1-TEL%129%NEB-SF/NEB-FF1%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%80/49</t>
+    <t>PE 367%STATISTICS FOR PETROLEUM ENGINEERS%Adjei Stephen%ED3-PE%82%NEB-TF%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%82</t>
+  </si>
+  <si>
+    <t>BME 463%BIOMATERIALS II%Agyapong Dorothy Araba Yakoba%ED4-BME%84%NEB-TF%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%84</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Oppong Tawiah Peter%ED1-TEL%129%VSLA/LT/303/206/N2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/25/20/14</t>
   </si>
   <si>
     <t>GE 263%INFORMATION SCIENCE AND PROGRAMMING%Tienaah Titus%ED2-GEOM%134%NEB-SF/NEB-FF1%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/50</t>
   </si>
   <si>
+    <t>ME 255%STRENGTH OF MATERIALS I%Andoh Prince Yaw%ED2-ME%242%Computer Based%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%242</t>
+  </si>
+  <si>
+    <t>ME 255%STRENGTH OF MATERIALS I%Andoh Prince Yaw%ED2-PE%97%Computer Based%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%97</t>
+  </si>
+  <si>
     <t>ME 255%STRENGTH OF MATERIALS I%Agyei Agyemang Anthony%ED2-AERO%74%NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/24</t>
   </si>
   <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Andoh Prince Yaw%ED2-ME%242%PB001/PB020/PB014/PB201/PB214/PB212%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45/45/20</t>
-  </si>
-  <si>
     <t>ME 255%STRENGTH OF MATERIALS I%Boahen Samuel%ED2-AE%155%NAF1/EA/A110/ECR/VCR%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/30/30/25/25</t>
   </si>
   <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED1-CE%32%304/N2%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/12</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED1-GEOL%34%303/N1%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30/14</t>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED1-CE%32%PB014%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%32</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED1-GEOL%34%PB020%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%34</t>
   </si>
   <si>
     <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-MSE%13%303%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%13</t>
   </si>
   <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-BME%17%PB208%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%17</t>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-BME%17%PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%17</t>
   </si>
   <si>
     <t>ECON 151%INTRODUCTION TO ECONOMICS %Takyi Paul Owusu%ED1-AUTO%88%VSLA/LT/206%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/26/17</t>
@@ -911,22 +896,22 @@
     <t>ECON 151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED2-EE%142%NAF1/EA/A110/ECR/VCR%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/30/30/20/20</t>
   </si>
   <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-TEL%30%PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30</t>
-  </si>
-  <si>
-    <t>ECON 151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED2-COE%36%RMA/RMB%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%18/18</t>
-  </si>
-  <si>
-    <t>ECON151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED3-GEOM%16%PB208%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%16</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED3-PCE%26%PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%26</t>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-TEL%30%303%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30</t>
+  </si>
+  <si>
+    <t>ECON 151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED2-COE%36%PB001%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%36</t>
+  </si>
+  <si>
+    <t>ECON151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED3-GEOM%16%PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%16</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED3-PCE%26%PB214%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%26</t>
   </si>
   <si>
     <t>ECON 151%INTRODUCTION TO ECONOMICS I%Takyi Paul Owusu%ED3-ME%230%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%85/80/45/20</t>
   </si>
   <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED3-CHE%32%304/N2%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/12</t>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED3-CHE%32%PB201%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/12</t>
   </si>
   <si>
     <t>ECON 151%INTRODUCTION TO ECONOMICS I%Takyi Paul Owusu%ED3-AERO%76%VSLA/LT%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/26</t>
@@ -938,7 +923,7 @@
     <t>IE 357%PROJECT MANAGEMENT%Asiedu Charlotte%ED3-IND%72%RMA/RMB/206%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%24/24/24</t>
   </si>
   <si>
-    <t>CE 451%STRUCTURAL ENGINEERING I%Osei Jack Banahene%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB212%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45/45/20</t>
+    <t>CE 451%STRUCTURAL ENGINEERING I%Osei Jack Banahene%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB208/PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/40/40/40/40/30/15</t>
   </si>
   <si>
     <t>COE 281%PROGRAMMING AND PROBLEM SOLIVING%Adjaidoo Theresa-Samuelle Maame Atwemaah%ED2-COE%253%Computer Based%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%253</t>
@@ -953,7 +938,7 @@
     <t>MSE 255%ELECTRICAL AND MAGNETIC BEHAVIOUR OF MATERIALS%Dzikunu Perseverance%ED2-MSE%80%NEB-TF/NEB-FF2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%60/20</t>
   </si>
   <si>
-    <t>MSE 255%ELECTRICAL AND MAGNETIC BEHAVIOUR OF MATERIALS%Nartey Martinson Addo%ED2-METE%59%NEB-SF%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%59</t>
+    <t>MSE 255%ELECTRICAL AND MAGNETIC BEHAVIOUR OF MATERIALS%Dzikunu Perseverance%ED2-METE%59%NEB-SF%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%59</t>
   </si>
   <si>
     <t>CE 151%ELEMENTARY STRUCTURES%Afrifa Russel Owusu%ED1-GEOL%119%VSLA/LT/303/RMA%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%50/30/20/20</t>
@@ -989,19 +974,16 @@
     <t>CHE 261%COMPUTER APPLICATIONS FOR ENGINEERS%Anang Daniel Adjah%ED2-CHE%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/30/30/25/25</t>
   </si>
   <si>
-    <t>CE 151%ELEMENTARY STRUCTURES%Afrifa Russel Owusu%ED1-CE%242%PB001/PB020/PB014/PB201/PB214/PB212%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/45/45/20</t>
-  </si>
-  <si>
-    <t>MSE 155%PRINCIPLES OF MATERIALS SCIENCE%Nartey Martinson Addo%ED1-METE%72%VSLA/RMA%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/22</t>
-  </si>
-  <si>
-    <t>MSE 155%PRINCIPLES OF MATERIALS SCIENCE%Nartey Martinson Addo%ED1-MSE%98%304/N1/RMB/206%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%25/25/24/24</t>
+    <t>CE 151%ELEMENTARY STRUCTURES%Afrifa Russel Owusu%ED1-CE%242%PB001/PB020/PB014/PB201/PB214/PB208%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/45/45/20</t>
+  </si>
+  <si>
+    <t>MSE 155%PRINCIPLES OF MATERIALS SCIENCE%Nartey Martinson Addo%ED1-MSE%98%PB208/PB008/PB214%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/30/38</t>
   </si>
   <si>
     <t>ME 365%THERMODYNAMICS  II%Forson Francis Kofi%ED3-AE%105%NAF1/EA/A110/ECR%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/25/20/20</t>
   </si>
   <si>
-    <t>ME 365%THERMODYNAMICS  II%Forson Francis Kofi%ED3-ME%230%PB001/PB020/PB014/PB201/PB214/PB212%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/40/40/40/20</t>
+    <t>ME 365%THERMODYNAMICS  II%Forson Francis Kofi%ED3-ME%230%PB001/PB020/PB014/PB201/PB008/PB212%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/42/43/30/25</t>
   </si>
   <si>
     <t>CE 463%WATER AND WASTE WATER ENGINEERING%Buamah Richard Akwasi%ED4-CE%245%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%85/85/52/23</t>
@@ -1010,7 +992,7 @@
     <t>COE 281%PROGRAMMING AND PROBLEM SOLIVING%Adjei Prince Ebenezer%ED2-BME%87%VSLA/LT/RMA%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/21/21</t>
   </si>
   <si>
-    <t>TE 251%ANALOG COMMUNICATION SYSTEMS%Affum Emmanuel Ampoma%ED2-TEL%179%NEB-TF/NEB-SF/NEB-FF2%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%80/80/20</t>
+    <t>TE 251%ANALOG COMMUNICATION SYSTEMS%Affum Emmanuel Ampoma%ED2-TEL%179%VSLA/RMA/303/304/N1/N2/206%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/20/30/22/25/20/17</t>
   </si>
   <si>
     <t>METE 351%PRINCIPLES OF HYDROMETALLURGY%Koomson Bennetta%ED3-METE%83%303/LT/RMB%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/30/23</t>
@@ -1019,10 +1001,10 @@
     <t>MSE 355%POLYMER PROCESSING%Asare Eric Kwame Anokye%ED3-MSE%89%304/N1/RMB/206%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%25/25/20/20</t>
   </si>
   <si>
-    <t>CHE 455%PROCESS CONTROL AND INSTRUMENTATION%Baidoo Martina Francisca%ED4-PCE%62%303/N2%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/32</t>
-  </si>
-  <si>
-    <t>PE 357%PETROLEUM PRODUCTION ENGINEERING I%Sarkodie Kwame%ED3-PE%82%PB008/PB208%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%41/41</t>
+    <t>CHE 455%PROCESS CONTROL AND INSTRUMENTATION%Baidoo Martina Francisca%ED4-PCE%62%NEB-TF%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%62</t>
+  </si>
+  <si>
+    <t>PE 357%PETROLEUM PRODUCTION ENGINEERING I%Sarkodie Kwame%ED3-PE%82%NEB-SF%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%82</t>
   </si>
   <si>
     <t xml:space="preserve">ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Ayetor Godwin Kafui Kwesi%ED2-MARI%37%Computer Based %Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%Computer Based </t>
@@ -1130,7 +1112,7 @@
     <t>COE 475%COMPUTER NETWORKING%Akowuah Emmanuel Kofi%ED4-COE%170%Computer Based%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%170</t>
   </si>
   <si>
-    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-AERO%74%PB201/PB208/PB008%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%30/30/24</t>
+    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-AERO%74%PB201/PB208/PB212%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/14</t>
   </si>
   <si>
     <t>ME 261%ENGINEERING MECHANICS II: DYNAMICS%Ampofo Joshua%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/80/50/27</t>
@@ -1166,10 +1148,13 @@
     <t>TE 271%ANALOG COMMUNICATION SYSTEMS%Ellis Sani Mubarak%ED3-EE%254%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/85/55/29</t>
   </si>
   <si>
+    <t>CHE 371%NATURAL GAS PROCESSING TECHNOLOGY%Benjamin Asante%ED3-CHE%50%PB208/PB008%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25</t>
+  </si>
+  <si>
     <t>TE 453%MOBILE AND WIRELESS COMMUNICATIONS%Agyekum Kwame Agyeman-Prempeh%ED4-TEL%142%PB001/PB020/PB014/PB212%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/40/42/15</t>
   </si>
   <si>
-    <t>ME 361%DYNAMICS OF MACHINERY%Ampofo Joshua%ED3-MARI%40%N1/206%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20</t>
+    <t>ME 361%DYNAMICS OF MACHINERY%Ampofo Joshua%ED3-MARI%40%N2/206%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20</t>
   </si>
   <si>
     <t>ME 361%DYNAMICS OF MACHINERY%Ampofo Joshua%ED3-AUTO%47%A110/ECR%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/22</t>
@@ -1181,46 +1166,46 @@
     <t>GE 371%SURVEY ADJUSTMENT I%Fosu Collins%ED3-GEOM%115%Computer Based%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%115</t>
   </si>
   <si>
-    <t>GE 271%ENGINEERING SURVEYING I%Arko-Adjei Anthony%ED2-GEOM%134%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/25/30/20/20</t>
+    <t>GE 271%ENGINEERING SURVEYING I%Arko-Adjei Anthony%ED2-GEOM%134%PB214/PB212/PB208/PB008%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/29/30/30</t>
   </si>
   <si>
     <t>CHE 251%CHEMICAL PROCESS CALCULATIONS I%Rockson Mizpah Ama Dziedzorm%ED2-CHE%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/30/30/25/25</t>
   </si>
   <si>
-    <t>CHE 251%CHEMICAL PROCESS CALCULATIONS I%Ohemeng-Boahen Godfred%ED2-PCE%59%PB008/PB208%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30/29</t>
-  </si>
-  <si>
-    <t>ARC 155%CLIMATE AND ARCHITECTURE%Amos-Abanyie Samuel%ED1-CE%74%PB008/PB208/PB212%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30/30/14</t>
-  </si>
-  <si>
-    <t>PE 359%RESERVOIR PETROPHYSICS%Erzuah Samuel%ED3-PE%82%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%52/30</t>
-  </si>
-  <si>
-    <t>CE 479%ENGINEERING AND ENVIRONMENTAL GEOPHYSICS%Owusu-Nimo Frederick%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB212%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45/45/20</t>
-  </si>
-  <si>
-    <t>PE 451%PETROLEUM ECONOMICS%Quaye Jonathan Atuquaye%ED4-PE%103%VSLA/LT/303%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/26/27</t>
-  </si>
-  <si>
-    <t>PE 255%FLUID MECHANICS%Adjei Stephen%ED2-PE%97%304/N1/RMB/206/N2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/20/20/20/17</t>
-  </si>
-  <si>
-    <t>TE 253%DIGITAL SYSTEMS%Obour Agyekum Kwame Opuni-Boachie%ED2-TEL%179%NEB-TF/NEB-SF/NEB-FF2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/80/19</t>
-  </si>
-  <si>
-    <t>TE 355%SIGNALS AND SYSTEMS%Agyekum Kwame Agyeman-Prempeh%ED3-TEL%147%NEB-TF/NEB-SF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/67</t>
-  </si>
-  <si>
-    <t>PCE 357%ORGANIC AND PETROCHEMICAL SYNTHESIS%Mensah Mary%ED3-PCE%51%NEB-FF1%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%51</t>
-  </si>
-  <si>
-    <t>CE 353%REINFORCED CONCRETE DESIGN%Owusu Twumasi Jones%ED3-CE%223%PB001/PB020/PB014/PB201/PB214%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45/43</t>
-  </si>
-  <si>
-    <t>GE 161%BASIC SURVEY PRINCIPLES I%Ayer John Wise Divine%ED1-GEOM%100%VSLA/LT/303%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/26/24</t>
-  </si>
-  <si>
-    <t>GE 475%RESEARCH METHODS%Duker Alfred Alan%ED4-GEOM%93%304/N1/RMB/206/N2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/20/20/20/13</t>
+    <t>CHE 251%CHEMICAL PROCESS CALCULATIONS I%Ohemeng-Boahen Godfred%ED2-PCE%59%PB208/PB008%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30/29</t>
+  </si>
+  <si>
+    <t>ARC 155%CLIMATE AND ARCHITECTURE%Amos-Abanyie Samuel%ED1-CE%74%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/24</t>
+  </si>
+  <si>
+    <t>PE 359%RESERVOIR PETROPHYSICS%Erzuah Samuel%ED3-PE%82%NEB-SF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%82</t>
+  </si>
+  <si>
+    <t>CE 479%ENGINEERING AND ENVIRONMENTAL GEOPHYSICS%Owusu-Nimo Frederick%ED4-CE%245%VSLA/LT/RMA/RMB/303/304/206/N1/N2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/25/24/24/30/21/24/25/22</t>
+  </si>
+  <si>
+    <t>PE 451%PETROLEUM ECONOMICS%Quaye Jonathan Atuquaye%ED4-PE%103%NEB-SF/NEB-FF2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/23</t>
+  </si>
+  <si>
+    <t>PE 255%FLUID MECHANICS%Adjei Stephen%ED2-PE%97%NEB-TF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%97</t>
+  </si>
+  <si>
+    <t>TE 253%DIGITAL SYSTEMS%Obour Agyekum Kwame Opuni-Boachie%ED2-TEL%179%PB001/PB020/PB014/PB201%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45</t>
+  </si>
+  <si>
+    <t>TE 355%SIGNALS AND SYSTEMS%Agyekum Kwame Agyeman-Prempeh%ED3-TEL%147%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/30/30/21/21</t>
+  </si>
+  <si>
+    <t>PCE 357%ORGANIC AND PETROCHEMICAL SYNTHESIS%Mensah Mary%ED3-PCE%51%NEB-TF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%51</t>
+  </si>
+  <si>
+    <t>CE 353%REINFORCED CONCRETE DESIGN%Owusu Twumasi Jones%ED3-CE%223%PB001/PB020/PB014/PB201/PB214/PB212%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%41/42/40/40/40/20</t>
+  </si>
+  <si>
+    <t>GE 161%BASIC SURVEY PRINCIPLES I%Ayer John Wise Divine%ED1-GEOM%100%VSLA/LT/RMA/RMB%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/20/20/20</t>
+  </si>
+  <si>
+    <t>GE 475%RESEARCH METHODS%Duker Alfred Alan%ED4-GEOM%93%303/304/206/N1/N2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%25/18/18/18/14</t>
   </si>
   <si>
     <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sackey Michael Nii%ED1-AERO%70%NAF1/A110%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%42/28</t>
@@ -1229,16 +1214,16 @@
     <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sackey Michael Nii%ED1-ME%223%VSLA/LT/303/304/N1/RMA/RMB/206/N2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%44/26/26/22/22/21/21/21/20</t>
   </si>
   <si>
-    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sekyere Charles Kofi Kafui%ED1-MARI%46%PB214/PB008%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%30/16</t>
-  </si>
-  <si>
-    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sekyere Charles Kofi Kafui%ED1-IND%81%NAF1/A110%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%48/33</t>
-  </si>
-  <si>
-    <t>EE 271%SEMICONDUCTOR DEVICES%Sekyere Yaw Opoku Mensah%ED2-EE%376%PB001/PB020/PB014/PB201/PB214/PB008/PB208/PB212%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%50/50/54/54/60/44/53/11</t>
-  </si>
-  <si>
-    <t>COE 271%SEMICONDUCTOR DEVICES%Kommey Benjamin%ED2-BME%87%PB001/PB020/PB212%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/40/7</t>
+    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sekyere Charles Kofi Kafui%ED1-MARI%46%A110/VCR%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%23/23</t>
+  </si>
+  <si>
+    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sekyere Charles Kofi Kafui%ED1-IND%81%303/304/206/RMB%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%25/20/20/20</t>
+  </si>
+  <si>
+    <t>EE 271%SEMICONDUCTOR DEVICES%Sekyere Yaw Opoku Mensah%ED2-EE%340%PB001/PB014/PB020/PB201/PB214/PB008/PB208/PB212/EA%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/45/45/45/45/30/30/25/30</t>
+  </si>
+  <si>
+    <t>COE 271%SEMICONDUCTOR DEVICES%Kommey Benjamin%ED2-BME%87%VSLA/LT/RMA%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/27/21</t>
   </si>
   <si>
     <t>COE 271%SEMICONDUCTOR DEVICES%Kommey Benjamin%ED2-COE%253%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%85/85/55/28</t>
@@ -1247,10 +1232,10 @@
     <t>EE 371%LINEAR ELECTRONIC CIRCUITS%Sekyere Yaw Opoku Mensah%ED3-EE%254%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%85/85/55/29</t>
   </si>
   <si>
-    <t>IE 365%ENGINEERING WORK STUDY%Takyi Gabriel%ED3-IND%72%PB014/PB020%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%36/36</t>
-  </si>
-  <si>
-    <t>EE 153%ELECTRICAL ENGINEERING TECHNOLOGY WITH MATLAB%Prah II Nicholas Kwesi%ED1-EE%287%VSLA/LT/303/304/N1/RMA/RMB/206/N2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%56/34/34/28/28/27/27/27/26</t>
+    <t>IE 365%ENGINEERING WORK STUDY%Takyi Gabriel%ED3-IND%72%NAF1/EA%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%44/28</t>
+  </si>
+  <si>
+    <t>EE 153%ELECTRICAL ENGINEERING TECHNOLOGY WITH MATLAB%Prah II Nicholas Kwesi%ED1-EE%287%PB001/PB014/PB020/PB201/PB214/PB208/PB008/PB212%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%42/42/42/42/42/30/28/20</t>
   </si>
   <si>
     <t>GED 151%BASIC GEOLOGY%Gawu Simon Kafui Yawo%ED1-GEOL%119%VSLA/RMA/303/N2%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/30/24/15</t>
@@ -1271,19 +1256,19 @@
     <t>CHE 253%CHEMICAL ENGINEERING THERMODYNAMICS I%Dogbe Eunice Sefakor Aku%ED2-PCE%59%NAF1/A110%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%39/20</t>
   </si>
   <si>
-    <t>AERO 391%AEROSPACE INDUSTRY AND ENGINEERING%K. K. Bofah%ED3-AERO%76%303/N1/206%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/25/21</t>
+    <t>AERO 391%AEROSPACE INDUSTRY AND ENGINEERING%K. K. Bofah%ED3-AERO%76%NEB-TF%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/25/21</t>
   </si>
   <si>
     <t>MSE 253%MECHANICAL BEHAVIOUR OF MATERIALS%Kwofie Samuel%ED2-MSE%80%LT/N1/RMB%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/25/25</t>
   </si>
   <si>
-    <t>MSE 253%MECHANICAL BEHAVIOUR OF MATERIALS%Kwofie Samuel%ED2-METE%59%NAF1/EA%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%39/20</t>
+    <t>MSE 253%MECHANICAL BEHAVIOUR OF MATERIALS%Kwofie Samuel%ED2-METE%59%303/N1/206%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%20/20/19</t>
   </si>
   <si>
     <t>GE 251%PRINCIPLES OF PHOTOGRAMMETRY%Ahorsu Harriet Atsufui%ED2-GEOM%134%PB020/PB201/PB008/PB212%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/30/14</t>
   </si>
   <si>
-    <t>CE 153%ENGINEERING PRACTICE AND TECHNOLOGY%Acquaah Vincent Kofi Abaka%ED1-CE%242%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%85/85/55/17</t>
+    <t>CE 153%ENGINEERING PRACTICE AND TECHNOLOGY%Acquaah Vincent Kofi Abaka%ED1-CE%242%NEB-SF/NEB-FF1/NEB-FF2/NAF1/EA/VCR%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%80/50/20/40/30/25</t>
   </si>
   <si>
     <t>CE 251%STRENGTH OF MATERIALS%Amponsah Evans%ED2-CE%260%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%85/85/55/35</t>
@@ -1292,6 +1277,9 @@
     <t>CE 251%STRENGTH OF MATERIALS%Kankam Charles Kwame%ED2-GEOL%154%PB001/PB014/PB214/PB208%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/19</t>
   </si>
   <si>
+    <t>CHE 363%POLYMER TECHNOLOGY%Boakye Patrick%ED3-CHE%36%ECR/VCR%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%25/11</t>
+  </si>
+  <si>
     <t>CHE 363%POLYMER TECHNOLOGY%Boakye Patrick%ED3-PCE%51%A110/EA%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%31/20</t>
   </si>
   <si>
@@ -1313,7 +1301,7 @@
     <t>MSE 457%METALWORKING PROCESSES%Kwofie Samuel%ED4-MSE%64%304/RMA/N2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%25/24/15</t>
   </si>
   <si>
-    <t>MSE 457%METAL FORMING PROCESSES%Kwofie Samuel%ED4-METE%49%NAF1%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%49</t>
+    <t>MSE 457%METAL FORMING PROCESSES%Kwofie Samuel%ED4-METE%49%A110/ECR%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%30/19</t>
   </si>
   <si>
     <t>CHE 463%ELECTROCHEMICAL TECHNOLOGY%Anang Daniel Adjah%ED4-PCE%18%A110%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%18</t>
@@ -1322,7 +1310,7 @@
     <t>CHE 463%ELECTROCHEMICAL TECHNOLOGY%Anang Daniel Adjah%ED4-CHE%40%NAF1%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40</t>
   </si>
   <si>
-    <t>CE 477%GEOTECHNICAL ENGINEERING I%Ayeh Felix Jojo Fianko%ED4-CE%245%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%85/85/57/18</t>
+    <t>CE 477%GEOTECHNICAL ENGINEERING I%Ayeh Felix Jojo Fianko%ED4-CE%245%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%80/80/55/30</t>
   </si>
   <si>
     <t>CE 477%GEOTECHNICAL ENGINEERING I%Ampadu Samuel Innocent Kofi%ED4-GEOL%102%LT/303/RMA/206%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%30/30/24/18</t>
@@ -1337,115 +1325,121 @@
     <t>ME 161%BASIC MECHANICS%Amoabeng Kofi Owura%ED1-BME%136%VSLA/LT/304/RMB/N2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%50/30/25/24/7</t>
   </si>
   <si>
-    <t>MME 473%MARINE MACHINERY SYSTEM DESIGN%Sackey Michael Nii%ED4-MARI%23%A110%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%23</t>
-  </si>
-  <si>
-    <t>COE 253%DISCRETE STRUCTURES%Kwabi Prince Amponsah%ED2-COE%253%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%85/85/57/26</t>
-  </si>
-  <si>
-    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-AERO%74%303/N1/RMB%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/25/19</t>
-  </si>
-  <si>
-    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-ME%242%VSLA/LT/303/304/N1/RMA/RMB/206%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/30/30/25/25/24/29/29</t>
-  </si>
-  <si>
-    <t>ME 451%BEHAVIOUR OF REAL FLUIDS%Opoku Richard%ED4-ME%144%VSLA/LT/304/RMA/206%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/30/25/24/15</t>
-  </si>
-  <si>
-    <t>ME 451%BEHAVIOUR OF REAL FLUIDS%Opoku Richard%ED4-AERO%61%NAF1/EA%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/16</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-MSE%98%PB020/PB201/PB212%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/54/8</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-TEL%129%PB001/PB014/PB214%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/45/39</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-MARI%46%A110/EA%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/16</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-ME%223%NEB-SF/NEB-TF/NEB-FF1%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%85/85/53</t>
-  </si>
-  <si>
-    <t>SES 171%FUNDAMENTALS OF ACQUATIC SKILLS%Afrifa Daniel%ED2-MARI%40%A110/VCR%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/10</t>
-  </si>
-  <si>
-    <t>AME 371%LAND VEHICLE DESIGN%Ayetor Godwin Kafui Kwesi%ED3-AUTO%47%NAF1/VCR%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%37/10</t>
-  </si>
-  <si>
-    <t>EE 261%DC MACHINES%Effah Francis Boafo%ED2-EE%376%PB001/PB020/PB014/PB201/PB214/PB008/PB208/PB212%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/45/45/45/51/52/60/33</t>
-  </si>
-  <si>
-    <t>IE 363%PROCESS PLANNING SYSTEMS%Sackey Samuel Mensah%ED3-IND%72%303/N1/RMB%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%30/25/17</t>
-  </si>
-  <si>
-    <t>MSE 363%MATERIALS CHARACTERIZATION TECHNIQUE%Arthur Emmanuel Kwesi%ED3-METE%83%NEB-TF/NEB-FF2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%60/23</t>
-  </si>
-  <si>
-    <t>MSE 363%MATERIALS CHARACTERIZATION TECHNIQUE%Arthur Emmanuel Kwesi%ED3-MSE%89%NAF1/EA/ECR%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/20/29</t>
-  </si>
-  <si>
-    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-COE%276%VSLA/LT/303/304/N1/RMA/RMB/206/N2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%50/30/30/25/25/24/31/30/31</t>
-  </si>
-  <si>
-    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-BME%94%NAF1/A110/VCR/ECR%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/20/20/14</t>
-  </si>
-  <si>
-    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-EE%254%PB001/PB020/PB014/PB201/PB214/PB208%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/45/44/30</t>
-  </si>
-  <si>
-    <t>CHE 351%MASS TRANSFER PROCESSES%Ankudey Emmanuel Godwin%ED3-CHE%100%PB001/PB020/PB008%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/40/20</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Boahen Samuel%ED1-GEOL%119%NEB-SF/NEB-FF1%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%69/50</t>
-  </si>
-  <si>
-    <t>BME 265%BIOLOGICAL TRANSPORT PHENOMENA%Odame Prince%ED2-BME%87%A110/EA/VCR/ECR%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20/20/27</t>
+    <t>MME 473%MARINE MACHINERY SYSTEM DESIGN%Sackey Michael Nii%ED4-MARI%23%ECR%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%23</t>
+  </si>
+  <si>
+    <t>COE 253%DISCRETE STRUCTURES%Kwabi Prince Amponsah%ED2-COE%253%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%85/85/53/30</t>
+  </si>
+  <si>
+    <t>ME 451%BEHAVIOUR OF REAL FLUIDS%Opoku Richard%ED4-ME%144%NAF1/EA/A110/VCR/ECR%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/30/30/25/20</t>
+  </si>
+  <si>
+    <t>ME 451%BEHAVIOUR OF REAL FLUIDS%Opoku Richard%ED4-AERO%61%RMA/RMB/206%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%21/20/20</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-MSE%98%PB201/PB208/PB212%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%43/30/25</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-TEL%129%PB001/PB014/PB020%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%43/43/43</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-MARI%46%N2/206%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%23/23</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-ME%223%VSLA/LT/303/304/RMA/RMB/N1/N2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/24/24/24/24/23</t>
+  </si>
+  <si>
+    <t>SES 171%FUNDAMENTALS OF ACQUATIC SKILLS%Afrifa Daniel%ED2-MARI%40%PB214%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40</t>
+  </si>
+  <si>
+    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-ME%242%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%81/81/50/30</t>
+  </si>
+  <si>
+    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-AERO%74%NAF1/A110%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%44/30</t>
+  </si>
+  <si>
+    <t>ME 251%FLUID MECHANICS I%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-AE%155%VSLA/LT/303/N1/304%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25/24</t>
+  </si>
+  <si>
+    <t>AME 371%LAND VEHICLE DESIGN%Ayetor Godwin Kafui Kwesi%ED3-AUTO%47%VCR/ECR%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%24/23</t>
+  </si>
+  <si>
+    <t>EE 261%DC MACHINES%Effah Francis Boafo%ED2-EE%340%PB001/PB014/PB020/PB201/PB214/PB008/PB208/PB212/EA%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/45/45/45/45/30/30/25/30</t>
+  </si>
+  <si>
+    <t>IE 363%PROCESS PLANNING SYSTEMS%Sackey Samuel Mensah%ED3-IND%72%ECR/VCR/A110%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25/22</t>
+  </si>
+  <si>
+    <t>MSE 363%MATERIALS CHARACTERIZATION TECHNIQUE%Arthur Emmanuel Kwesi%ED3-METE%83%RMA/RMB/N1/206%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%21/21/21/20</t>
+  </si>
+  <si>
+    <t>MSE 363%MATERIALS CHARACTERIZATION TECHNIQUE%Arthur Emmanuel Kwesi%ED3-MSE%89%NEB-TF/NEB-FF2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%64/25</t>
+  </si>
+  <si>
+    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-COE%276%PB001/PB020/PB014/PB201/PB214/PB008/PB212%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/45/45/30/21</t>
+  </si>
+  <si>
+    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-BME%94%NAF1/EA/VCR%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/24</t>
+  </si>
+  <si>
+    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-EE%254%PB001/PB020/PB014/PB201/PB214/PB208%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/45/45/29</t>
+  </si>
+  <si>
+    <t>CHE 351%MASS TRANSFER PROCESSES%Ankudey Emmanuel Godwin%ED3-CHE%100%NAF1/EA/A110%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Boahen Samuel%ED1-GEOL%119%VSLA/LT/303/304%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/25/24</t>
+  </si>
+  <si>
+    <t>BME 265%BIOLOGICAL TRANSPORT PHENOMENA%Odame Prince%ED2-BME%87%RMA/RMB/N1/N2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%22/22/22/21</t>
   </si>
   <si>
     <t>ME 159%TECHNICAL DRAWING%Boahen Samuel%ED1-PCE%56%PB208/PB008%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%28/28</t>
   </si>
   <si>
-    <t>ME 159%TECHNICAL DRAWING%Asante Eric Amoah%ED1-CHE%120%PB014/PB201/PB214%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/40/40</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Aveyire Joseph%ED1-CE%242%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/85/55/17</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Aveyire Joseph%ED1-AE%126%VSLA/LT/304/RMA%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%50/30/25/21</t>
-  </si>
-  <si>
-    <t>CE 359%SOIL MECHANICS%Charkley Frederick Nai%ED3-CE%223%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/80/52/11</t>
-  </si>
-  <si>
-    <t>GED 379%SOIL MECHANICS%Amenuvor Andrew Cudzo%ED3-GEOL%154%LT/RMA/RMB/VSLA/N2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30/24/24/50/26</t>
-  </si>
-  <si>
-    <t>PE 259%SURVIVAL SWIMMING TECHNIQUES%Gyamfi Isaac%ED2-PE%97%PB001/PB020/PB214%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/40/17</t>
-  </si>
-  <si>
-    <t>PCE 451%CATALYSIS%Baidoo Martina Francisca%ED4-PCE%62%VCR/ECR/NAF1%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%25/25/12</t>
-  </si>
-  <si>
-    <t>ME 373%MACHINE ELEMENTS DESIGN I%Davis Francis%ED3-ME%230%PB001/PB020/PB014/PB008/PB201/PB214%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/30/45/20</t>
-  </si>
-  <si>
-    <t>ME 455%FINITE ELEMENT METHODS%Andoh Prince Yaw%ED4-ME%144%VCR/ECR/A110/EA/NAF1%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%24/24/29/29/38</t>
-  </si>
-  <si>
-    <t>GE 351%STEREO PHOTOGRAMMETRY%Tienaah Titus%ED3-GEOM%115%PB014/PB008/PB201/PB214%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/25/40/10</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Tay Godwin Fabiola Kwaku%ED1-COE%261%LT/RMA/RMB/VSLA/206/303/304/N1/N2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30/24/24/50/24/30/28/29/22</t>
-  </si>
-  <si>
-    <t>AME 485%AUTOMATIC POWER TRAIN%Abu Frimpong Solomon%ED4-AUTO%32%304/N1%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%16/16</t>
-  </si>
-  <si>
-    <t>CE 461%ENG ECONOMY AND ENTERPRENEURSHIP DEVELOPMENT%Appiah-Effah Eugene%ED4-GEOM%93%A110/EA/NAF1%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30/30/33</t>
-  </si>
-  <si>
-    <t>CE 461%ENGINEERING ECONOMY AND ENTERPRENEURSHIP%Appiah-Effah Eugene%ED4-CE%245%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%87/87/54/17</t>
+    <t>ME 159%TECHNICAL DRAWING%Asante Eric Amoah%ED1-CHE%120%VSLA/LT/303/304%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30/20</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Aveyire Joseph%ED1-CE%242%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/85/50/22</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Aveyire Joseph%ED1-AE%126%NEB-SF/NEB-FF1%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%75/51</t>
+  </si>
+  <si>
+    <t>CE 359%SOIL MECHANICS%Charkley Frederick Nai%ED3-CE%223%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%75/75/50/23</t>
+  </si>
+  <si>
+    <t>GED 379%SOIL MECHANICS%Amenuvor Andrew Cudzo%ED3-GEOL%154%VSLA/LT/303/304/206%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%49/30/30/25/20</t>
+  </si>
+  <si>
+    <t>PE 259%SURVIVAL SWIMMING TECHNIQUES%Gyamfi Isaac%ED2-PE%97%VSLA/LT/303/304/206%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/25/20/12</t>
+  </si>
+  <si>
+    <t>PCE 451%CATALYSIS%Baidoo Martina Francisca%ED4-PCE%62%N1/RMA/RMB%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%22/20/20</t>
+  </si>
+  <si>
+    <t>ME 373%MACHINE ELEMENTS DESIGN I%Davis Francis%ED3-ME%230%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/80/50/20</t>
+  </si>
+  <si>
+    <t>GE 351%STEREO PHOTOGRAMMETRY%Tienaah Titus%ED3-GEOM%115%NAF1/EA/A110/VCR%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/30/30/15</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Tay Godwin Fabiola Kwaku%ED1-COE%261%PB001/PB020/PB014/PB201/PB214/PB208/PB212%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%42/42/42/42/42/30/21</t>
+  </si>
+  <si>
+    <t>MME 365%ENGINEERING THERMODYNAMICS%Amoabeng Kofi Owura%ED3-MARI%40%ECR/VCR%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/20</t>
+  </si>
+  <si>
+    <t>AME 485%AUTOMATIC POWER TRAIN%Abu Frimpong Solomon%ED4-AUTO%32%RMA/RMB%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%16/16</t>
+  </si>
+  <si>
+    <t>CE 461%ENG ECONOMY AND ENTERPRENEURSHIP DEVELOPMENT%Appiah-Effah Eugene%ED4-GEOM%93%NAF1/EA/A110%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/25/28</t>
+  </si>
+  <si>
+    <t>CE 461%ENGINEERING ECONOMY AND ENTERPRENEURSHIP%Appiah-Effah Eugene%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB212%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45/45/20</t>
+  </si>
+  <si>
+    <t>ME 455%FINITE ELEMENT METHODS%Andoh Prince Yaw%ED4-ME%144%Computer Based%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%144</t>
   </si>
   <si>
     <t>GE 151%CARTOGRAPHY I%Quaye-Ballard Jonathan Arthur%ED1-GEOM%100%PB008/PB208/PB214/PB212%Monday, 23 February 2026%Session, 1 (8:15AM - 9:15 AM)%30/30/20/20</t>
@@ -1454,10 +1448,13 @@
     <t>GED 253%PHYSICAL GEOLOGY%Mensah Emmanuel%ED2-GEOL%154%PB014/PB001/PB020/PB008%Monday, 23 February 2026%Session, 1 (8:15AM - 9:15 AM)%40/44/40/30</t>
   </si>
   <si>
-    <t>MATH 151%ALGEBRA%Barnes Benedict%ED1-PCE%56%PB008/PB208%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/26</t>
-  </si>
-  <si>
-    <t>MME 365%ENGINEERING THERMODYNAMICS%Amoabeng Kofi Owura%ED3-MARI%40%206/303%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/20</t>
+    <t>CHE 255%FLUID TRANSPORT%Dogbe Eunice Sefakor Aku%ED2-PCE%59%PB214/PB201%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%30/29</t>
+  </si>
+  <si>
+    <t>GED 251%MINERALOGY%Wilson Matthew Coffie%ED2-GEOL%154%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%80/50/24</t>
+  </si>
+  <si>
+    <t>MSE 155%PRINCIPLES OF MATERIALS SCIENCE%Nartey Martinson Addo%ED1-METE%72%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/22</t>
   </si>
 </sst>
 </file>
@@ -1834,10 +1831,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A481"/>
+  <dimension ref="A1:A480"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="199.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="212.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -1952,7 +1949,7 @@
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
@@ -1977,7 +1974,7 @@
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
@@ -1997,2252 +1994,2247 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>477</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>93</v>
+        <v>478</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="147" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>479</v>
+        <v>147</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="201" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="202" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="203" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="204" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="205" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="206" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="209" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="210" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="211" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="212" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="213" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="214" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="215" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="216" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="217" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="218" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="219" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="220" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="221" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="222" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="223" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="224" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="226" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="227" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="228" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="229" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="239" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="241" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="242" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="246" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="248" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="252" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="253" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="256" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="257" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="259" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="260" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="261" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="262" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="263" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="264" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="265" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="266" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="267" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="268" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="269" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="270" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="271" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="272" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="273" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="274" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="275" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="276" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="277" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="278" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="279" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="280" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="281" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="282" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="283" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="284" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="285" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="286" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="287" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="288" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="289" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="290" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="291" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="292" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="293" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="294" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="295" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="296" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="297" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="298" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="299" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="300" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="301" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="302" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="303" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="304" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="305" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="306" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="307" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="308" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="309" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="310" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="311" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="312" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="313" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="314" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="315" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="316" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="317" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="318" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="319" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="320" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="321" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="322" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="323" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="324" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="325" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
-        <v>321</v>
+        <v>479</v>
       </c>
     </row>
     <row r="326" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="327" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="328" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="329" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="330" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="331" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="332" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="333" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="334" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="335" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="336" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="337" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="338" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="339" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="340" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="341" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="342" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="343" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="344" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="345" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A345" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="346" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="347" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A347" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="348" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="349" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A349" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="350" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A350" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="351" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="352" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="353" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A353" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="354" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A354" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="355" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A355" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="356" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A356" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="357" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="358" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="359" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="360" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="361" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="362" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
     </row>
     <row r="363" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="364" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="365" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="366" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
     </row>
     <row r="367" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="368" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="369" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="370" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A370" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="371" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A371" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="372" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A372" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="373" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A373" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="374" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A374" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
     </row>
     <row r="375" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A375" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="376" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A376" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
     </row>
     <row r="377" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A377" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="378" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="379" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="380" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="381" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="382" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="383" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A383" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="384" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="385" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A385" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="386" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A386" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="387" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A387" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
     </row>
     <row r="388" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A388" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="389" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A389" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="390" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A390" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="391" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A391" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="392" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A392" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="393" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A393" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="394" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="395" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="396" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A396" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="397" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A397" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="398" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A398" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="399" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A399" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="400" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="401" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="402" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="403" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A403" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="404" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A404" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="405" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="406" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="407" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A407" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="408" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A408" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="409" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A409" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="410" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="411" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A411" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="412" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A412" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="413" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A413" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="414" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="415" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="416" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A416" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="417" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A417" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="418" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A418" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="419" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A419" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="420" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A420" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="421" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A421" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="422" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A422" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="423" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A423" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="424" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A424" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="425" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A425" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="426" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A426" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="427" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A427" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="428" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A428" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="429" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A429" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="430" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A430" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="431" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A431" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="432" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A432" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="433" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A433" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="434" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="435" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="436" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A436" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="437" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="438" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A438" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="439" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A439" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="440" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A440" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="441" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A441" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="442" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="443" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A443" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="444" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A444" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="445" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A445" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="446" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A446" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="447" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A447" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="448" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A448" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
     </row>
     <row r="449" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A449" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="450" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A450" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="451" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A451" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
     <row r="452" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A452" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="453" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A453" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="454" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="455" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="456" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A456" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="457" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A457" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="458" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A458" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="459" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A459" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="460" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A460" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="461" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A461" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="462" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A462" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="463" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A463" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="464" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A464" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="465" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A465" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="466" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A466" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="467" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A467" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="468" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A468" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="469" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A469" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="470" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A470" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="471" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A471" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="472" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A472" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="473" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A473" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="474" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A474" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="475" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A475" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="476" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A476" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="477" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A477" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="478" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A478" t="s">
-        <v>480</v>
+        <v>472</v>
       </c>
     </row>
     <row r="479" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A479" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="480" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A480" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="481" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A481" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
worked on updated timetable
</commit_message>
<xml_diff>
--- a/src/outputs/Mid-Sem TT-cleaned.xlsx
+++ b/src/outputs/Mid-Sem TT-cleaned.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B09F45B6-89A3-40FC-8C3B-5C0799C20F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C17D2F4-C9F9-4729-8B99-A82DD63CB481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="477">
   <si>
     <t xml:space="preserve">MATH 351%NUMERICAL ANALYSIS%Azure Isaac%ED3-ME%230%Computer Based %Monday, 23 February 2026%Session, 1 (8:15AM - 9:15 AM)%Computer Based </t>
   </si>
@@ -107,15 +107,6 @@
     <t>CE 457%DRAINAGE SYSTEMS%Adjei Kwaku Amaning%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB212%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%45/45/45/45/45/20</t>
   </si>
   <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Dzebre Denis Edem Kwame%ED2-MARI%37%N1/N2%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%20/17</t>
-  </si>
-  <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Dzebre Denis Edem Kwame%ED2-AUTO%77%EA/ECR/VCR%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%30/25/22</t>
-  </si>
-  <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Dzebre Denis Edem Kwame%ED2-IND%80%303/304/206/RMB%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%22/20/20/18</t>
-  </si>
-  <si>
     <t>BME 471%BIOINSTRUMENTATION II%Acquah Isaac%ED4-BME%84%PB008/PB208/PB212%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%30/30/24</t>
   </si>
   <si>
@@ -455,1003 +446,1003 @@
     <t>MATH 151%ALGEBRA%Barnes Benedict%ED1-CHE%120%VSLA/LT/304/RMA%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%46/25/25/24</t>
   </si>
   <si>
+    <t>MATH 151%ALGEBRA%Adu-Ansah Lawton%ED1-TEL%129%VSLA/LT/304/RMA%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/30/25/24</t>
+  </si>
+  <si>
+    <t>MATH 151%ALGEBRA%Azure Isaac%ED1-AUTO%88%RMB/303/N1/N2%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%22/22/22/22</t>
+  </si>
+  <si>
+    <t>MATH 151%ALGEBRA%Ayekple Yao Elikem%ED1-EE%287%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2/NAF1%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%80/85/55/30/37</t>
+  </si>
+  <si>
+    <t>MATH 151%ALGEBRA%Azure Isaac%ED1-GEOM%100%RMB/303/N1/N2%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%22/30/24/24</t>
+  </si>
+  <si>
+    <t>TE 357%OPTICAL COMMUNICATION%Gadze James Dzisi%ED3-TEL%147%PB020/PB201/PB214/PB212%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/40/40/25</t>
+  </si>
+  <si>
+    <t>IE 355%DISCRETE EVENT SIMULATION%Takyi Gabriel%ED3-IND%72%VSLA/303%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%44/28</t>
+  </si>
+  <si>
+    <t>AE 457%CROP PROCESSING%Darko Joseph Ofei %ED4-AE%103%VSLA/LT/RMA/RMB%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/25/20/18</t>
+  </si>
+  <si>
+    <t>GED 459%EXPLORATION GEOCHEMISTRY%Gawu Simon Kafui Yawo%ED4-GEOL%102%LT/N1/RMA/RMB/N2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%22/22/20/20/20</t>
+  </si>
+  <si>
+    <t>CE 467%HIGHWAY ENGINEERING II%Tuffour Yaw Adubofour%ED4-CE%245%PB001/PB014/PB201/PB214/PB208/PB008/PB212%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%42/42/42/42/30/28/20</t>
+  </si>
+  <si>
+    <t>COE 485%COMPUTER ARCHITECTURE%Boateng Kwame Osei%ED4-COE%170%PB001/PB014/PB020/PB208/PB008%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/40/40/25/25</t>
+  </si>
+  <si>
+    <t>TE 481%WIRELESS DATA COMMUNICATION NETWORK%Opare Kwasi Adu-Boahen%ED4-EE%224%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%75/75/50/24</t>
+  </si>
+  <si>
+    <t>IE 459%RISK ANALYSIS%Asiedu Charlotte%ED4-IND%67%NAF1/EA%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/27</t>
+  </si>
+  <si>
+    <t>CE 355%HYDROLOGY%Adjei Kwaku Amaning%ED3-CE%223%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%75/75/50/23</t>
+  </si>
+  <si>
+    <t>PCE 455%POLLUTION CONTROL IN PETROCHEMICAL INDUSTRY%Kwao-Boateng Emmanuela%ED4-PCE%62%303/206/304%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%22/20/20</t>
+  </si>
+  <si>
+    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-MARI%23%ECR%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%23</t>
+  </si>
+  <si>
+    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-AUTO%32%N1/N2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%16/16</t>
+  </si>
+  <si>
+    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-ME%144%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%45/30/30/20/20</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Boateng Maxwell Akwasi%ED2-MARI%37%206/RMB%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%20/17</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Boateng Maxwell Akwasi%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%80/80/55/27</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-TEL%179%VSLA/LT/303/N1/N2/RMA%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/30/30/25/24/20</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-GEOL%154%VSLA/303/N1/RMA/RMB/304%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/25/25/20/20/20</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-COE%253%PB001/PB014/PB020/PB201/PB214/PB208/PB212%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/40/40/40/40/28/25</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-IND%80%EA/A110/VCR%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/20/20</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-AE%155%NEB-TF/NEB-SF%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%78/77</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-CE%260%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%42/42/42/42/42/25/25</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-AERO%74%NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/24</t>
+  </si>
+  <si>
+    <t>MATH 251%DIFFERENTIAL EQUATIONS%Barnes Benedict%ED2-GEOM%134%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/25/25/20/20</t>
+  </si>
+  <si>
+    <t>AERO 473%AEROSPACE VEHICLE DESIGN%Oppong David Kofi%ED4-AERO%61%NAF1/ECR%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/21</t>
+  </si>
+  <si>
+    <t>CHE 357%EXPERIMENTAL DATA ANALYSIS%Kwao-Boateng Emmanuela%ED3-PCE%51%PB008/PB212%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/21</t>
+  </si>
+  <si>
+    <t>CHE 357%EXPERIMENTAL DATA ANALYSIS%Rockson Mizpah Ama Dziedzorm%ED3-CHE%100%LT/206/N2/304%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/25/24/24</t>
+  </si>
+  <si>
+    <t>CE 155%ENVIRONMENTAL STUDIES%Appiah-Brempong Miriam%ED1-AERO%70%PB208/PB008/PB212%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25/20</t>
+  </si>
+  <si>
+    <t>CE 155%ENVIRONMENTAL STUDIES%Buamah Richard Akwasi%ED1-AE%126%VSLA/LT/303/304%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/30/30/21</t>
+  </si>
+  <si>
+    <t>CE 155%ENVIRONMENTAL STUDIES%Essandoh Helen Michelle Korkor%ED1-COE%261%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%42/42/42/42/42/28/25</t>
+  </si>
+  <si>
+    <t>CE 155%ENVIRONMENTAL STUDIES%Appiah-Brempong Miriam%ED1-IND%81%NEB-TF%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%81</t>
+  </si>
+  <si>
+    <t>CE 155%ENVIRONMENTAL STUDIES%Buamah Richard Akwasi%ED1-TEL%129%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30/22/20</t>
+  </si>
+  <si>
+    <t>CE 155%ENVIRONMENTAL STUDIES%Awuah Esi%ED1-ME%223%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%75/75/55/20</t>
+  </si>
+  <si>
+    <t>CHE 151%INORGANIC CHEMISTRY FOR ENGINEERS%Opoku Francis%ED1-CHE%120%PB001/PB014/PB020%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/40/40</t>
+  </si>
+  <si>
+    <t>CHE 151%INORGANIC CHEMISTRY FOR ENGINEERS%Opoku Francis%ED1-PCE%56%EA/A110%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%28/28</t>
+  </si>
+  <si>
+    <t>PE 151%INORGANIC CHEMISTRY FOR ENGINEERS%Opoku Francis%ED1-PE%129%VSLA/LT/303/N1%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/30/30/25</t>
+  </si>
+  <si>
+    <t>METE 453%METALLURGICAL FAILURE ANALYSIS AND NDTs%Arthur Emmanuel Kwesi%ED4-METE%49%206/304%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/24</t>
+  </si>
+  <si>
+    <t>MSE 455%FAILURE ANALYSIS AND NON-DESTRUCTIVE TESTING%Arthur Emmanuel Kwesi%ED4-MSE%64%RMA/RMB/N2%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%22/22/20</t>
+  </si>
+  <si>
+    <t>MSE 351%ENGINEERING CERAMICS%Andrews Anthony%ED3-MSE%89%NAF1/VCR/ECR%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/25/24</t>
+  </si>
+  <si>
+    <t>GED 351%PETROLOGY%Foli Gordon%ED3-GEOL%154%NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%80/50/30</t>
+  </si>
+  <si>
+    <t>GE 463%LAND AND GEOGRAPHIC INFORMATION SYSTEM I%Forkuo Eric Kwabena%ED4-GEOM%93%PB201/PB214/PB212%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/40/13</t>
+  </si>
+  <si>
+    <t>MME 373%DESIGN OF MARINE MACHINE ELEMENTS%Andoh Prince Yaw%ED3-MARI%40%Computer Based%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40</t>
+  </si>
+  <si>
+    <t>AME 373%DESIGN OF AUTO MECHANICAL SYSTEMS%Andoh Prince Yaw%ED3-AUTO%47%Computer Based%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%47</t>
+  </si>
+  <si>
+    <t>PCE 253%INTRODUCTION TO PETROCHEMICAL INDUSTRIES%Baidoo Martina Francisca%ED2-PCE%59%NEB-TF%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%59</t>
+  </si>
+  <si>
+    <t>CHE 259%CHEMICAL PROCESS INDUSTRIES%Afotey Benjamin%ED2-CHE%154%NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/50/24</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Adam Faisal Wahib%ED1-GEOL%119%NAF1/EA/A110/ECR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/27/27/20</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Opoku Richard%ED1-CE%242%VSLA/LT/303/304/RMA/RMB/206/N1/N2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/30/30/25/24/24/20/20/20</t>
+  </si>
+  <si>
+    <t>CE 367%HIGHWAY AND TRANSPORTATION ENGINEERING I%Ababio-Donkor Augustus%ED3-GEOM%115%VSLA/LT/303/304%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%43/26/26/20</t>
+  </si>
+  <si>
+    <t>EE 365%ELECTRICAL SERVICES DESIGN%Kwegyir Daniel%ED3-EE%254%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/40/40/40/40/30/24</t>
+  </si>
+  <si>
+    <t>CE 475%SYSTEMS ENGINEERING I%Donkor Emmanuel Amponsah%ED4-CE%245%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/80/55/30</t>
+  </si>
+  <si>
+    <t>TE 385%SIGNALS AND SYSTEMS%Yeboah-Akowuah Bright%ED3-COE%276%PB001/PB014/PB020/PB201/PB214/PB008/PB212%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45/45/30/21</t>
+  </si>
+  <si>
+    <t>TE 385%SIGNALS AND SYSTEMS%Yeboah-Akowuah Bright%ED3-BME%94%N1/N2/RMA/RMB%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%25/24/23/22</t>
+  </si>
+  <si>
+    <t>TE 463%AVIATION COMMUNICATION%Obeng Kwakye Kingsford Sarkodie%ED4-TEL%142%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/30/30/22/20</t>
+  </si>
+  <si>
+    <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-CHE%39%206/VCR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%24/15</t>
+  </si>
+  <si>
+    <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-PE%3%ECR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%3</t>
+  </si>
+  <si>
+    <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-PCE%45%PB208/PB212%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%25/20</t>
+  </si>
+  <si>
+    <t>ME 281%ENGINEERING MATERIALS I%Amoabeng Kofi Owura%ED2-AERO%74%A110/EA/VCR%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%28/28/18</t>
+  </si>
+  <si>
+    <t>ME 281%ENGINEERING MATERIALS I%Amoabeng Kofi Owura%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%80/80/55/27</t>
+  </si>
+  <si>
+    <t>AE 153%AGRIC. METEOROLOGY AND CLIMATOLOGY%Bessah Enoch%ED1-AE%126%NEB-SF/NEB-FF1%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%75/51</t>
+  </si>
+  <si>
+    <t>GED 365%GEOLOGICAL FIELD MAPPPING%Brako Blestmond Afrifa%ED3-GEOL%154%VSLA/LT/303/RMA/RMB/304%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/28/28/20/20/18</t>
+  </si>
+  <si>
+    <t>AME 455%VEHICLE AIR-CONDITIONING AND REFRIGERATION%Sekyere Charles Kofi Kafui%ED4-AUTO%32%N1/N2%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%16/16</t>
+  </si>
+  <si>
+    <t>SOC 255%INTRODDUCTION TO RURAL SOCIOLOGY%Boateng Kwabena%ED2-METE%59%N1/N2/206%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20/19</t>
+  </si>
+  <si>
+    <t>SOC 255%INTRODUCTION TO RURAL SOCIOLOGY%Boateng Kwabena%ED3-METE%83%NAF1/VCR/ECR%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/22/22</t>
+  </si>
+  <si>
+    <t>MME 465%MARINE AIR CONDITIONING AND REFRIGERATION%Sekyere Charles Kofi Kafui%ED4-MARI%23%206%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%23</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Dzebre Denis Edem Kwame%ED1-GEOM%100%NEB-TF/NEB-FF2%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%75/25</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Dzebre Denis Edem Kwame%ED1-EE%287%PB001/PB014/PB020/PB201/PB214/PB008/PB208/PB212%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%42/42/42/42/42/30/28/20</t>
+  </si>
+  <si>
+    <t>ME 465%AIR CONDITIONING AND REFRIGERATION%Sekyere Charles Kofi Kafui%ED4-AERO%61%NAF1/ECR%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/21</t>
+  </si>
+  <si>
+    <t>ME 465%AIR CONDITIONING AND REFRIGERATION%Sekyere Charles Kofi Kafui%ED4-ME%144%PB001/PB014/PB020/PB008%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/40/40/25</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Darko Jeel Pharis%ED3-CHE%64%303/206/304%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%24/20/20</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED1-CE%136%PB201/PB214/PB208/PB212%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/40/30/26</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED1-GEOL%80%RMB/N1/N2/304%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%20/20/20/20</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED2-BME%42%NAF1%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%42</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED2-COE%146%PB001/PB014/PB020/PB008%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/40/40/27</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED2-EE%174%VSLA/LT/303/N1/RMA/RMB%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/30/30/24/24/24</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Ocloo Alexander%ED2-MSE%53%NEB-FF1%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%53</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Ocloo Alexander%ED2-TEL%104%NEB-SF/NEB-FF2%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%80/24</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Osei-Danso Harriet Efua%ED3-GEOM%60%A110/EA%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/30</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED1-MARI%46%VCR/ECR%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%23/23</t>
+  </si>
+  <si>
+    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Darko Jeel Pharis%ED3-PCE%22%PB208%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%22</t>
+  </si>
+  <si>
+    <t>METE 151%INTRODUCTION TO METALLURGICAL ENGINEERING%Koomson Bennetta%ED1-METE%72%NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%47/25</t>
+  </si>
+  <si>
+    <t>AERO 157%INTRODUCTION TO AVIATION TECHNOLOGY%Oppong David Kofi%ED1-AERO%70%NEB-TF%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%70</t>
+  </si>
+  <si>
+    <t>CHEM 151%GENERAL CHEMISTRY%Sarpong Lilian%ED1-BME%136%NAF1/EA/A110/VCR/ECR%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/28/28/20/20</t>
+  </si>
+  <si>
+    <t>EE 371%MICROELECTRONIC CIRCUITS%Acheampong Francisca Adoma%ED3-TEL%147%NEB-SF/NEB-TF%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%74/73</t>
+  </si>
+  <si>
+    <t>COE 371%LINEAR ELECTRONIC CIRCUITS%Agbemenu Andrew Selasi%ED3-COE%276%PB001/PB014/PB020/PB201/PB214/PB008/PB212%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/45/45/30/21</t>
+  </si>
+  <si>
+    <t>COE 371%LINEAR ELECTRONIC CIRCUITS%Agbemenu Andrew Selasi%ED3-BME%94%VSLA/LT/RMA%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%42/28/24</t>
+  </si>
+  <si>
+    <t>CHE 257%ANALYTICAL CHEMISTRY FOR CHEMICAL ENGINEERS%Boakye Patrick%ED2-CHE%154%NEB-TF/NEB-SF%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%77/77</t>
+  </si>
+  <si>
+    <t>CHE 257%ANALYTICAL CHEMISTRY FOR CHEMICAL ENGINEERS%Boakye Patrick%ED2-PCE%59%A110/EA/VCR%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%20/20/19</t>
+  </si>
+  <si>
+    <t>ME 281%ENGINEERING MATERIALS I%Boahen Samuel%ED2-AUTO%77%NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%50/27</t>
+  </si>
+  <si>
+    <t>MME 281%MARINE ENGINEERING MATERIALS%Boahen Samuel%ED2-MARI%37%PB208/PB212%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%20/17</t>
+  </si>
+  <si>
+    <t>ME 281%ENGINEERING MATERIALS I%Boahen Samuel%ED2-IND%80%PB001/PB014%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/40</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sekyere Charles Kofi Kafui%ED1-AUTO%88%VSLA/303/304%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/30/18</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sekyere Charles Kofi Kafui%ED1-IND%81%NEB-SF%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%81</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Afriyie Nyarko Frank Kwabena%ED1-COE%261%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%42/42/42/42/42/26/25</t>
+  </si>
+  <si>
+    <t>PE 455%RESERVOIR SIMULATION%Ampomah William%ED4-PE%103%NEB-TF/NEB-FF2%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%78/25</t>
+  </si>
+  <si>
+    <t>GED 465%ENGINEERING GEOLOGICAL INVESTIGATIONS%Ali Bukari%ED4-GEOL%102%PB201/PB214/PB208%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/40/23</t>
+  </si>
+  <si>
+    <t>GE 281%BASIC PHYSICAL GEODESY%Dadzie Isaac%ED2-GEOM%134%VSLA/LT/303/RMA/RMB%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/27/27/22/22</t>
+  </si>
+  <si>
+    <t>PE 257%PETROLEUM ENGINEERING THERMODYNAMICS I%Sokama-Neuyam Yen Adams%ED2-PE%97%LT/N1/N2/206%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%25/24/24/24</t>
+  </si>
+  <si>
+    <t>CHE 451%CHEMICAL PROCESS DESIGN AND ECONOMICS%Afotey Benjamin%ED4-CHE%114%NAF1/EA/VCR/ECR%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/25/25/24</t>
+  </si>
+  <si>
+    <t>CHE 451%CHEMICAL PROCESS DESIGN AND ECONOMICS%Afotey Benjamin%ED4-PCE%62%N1/N2/RMA%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%22/20/20</t>
+  </si>
+  <si>
+    <t>METE 451%METALLURGICAL PLANT DESIGN/OPERATIONS%Koomson Bennetta%ED4-METE%49%NEB-FF1%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%49</t>
+  </si>
+  <si>
+    <t>IE 455%COSTING AND BREAK-EVEN ANALYSIS%Mensah Lena Dzifa%ED4-IND%67%PB020/PB212%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/27</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%Amoako-Yirenkyi Carole Fredua%ED3-ME%230%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%230</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%Amoako-Yirenkyi Carole Fredua%ED3-COE%276%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%276</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%Amoako-Yirenkyi Carole Fredua%ED3-IND%72%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%72</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%C. F. A. Yirenkyi%ED3-AERO%76%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%76</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%Amoako-Yirenkyi Carole Fredua%ED3-GEOM%93%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%93</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%Okutu John Kwadey%ED3-EE%254%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/40/40/40/40/27/27</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%David Benteh%ED3-MARI%40%PB212%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%David Benteh%ED3-GEOL%154%NAF1/EA/A110/VCR/ECR%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25/25</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%Okutu John Kwadey%ED3-AUTO%47%VCR/ECR%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%24/24</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%David Benteh%ED3-BME%94%NAF1/EA/A110%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/27/27</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%Benteh David%ED3-MSE%89%LT/N2/RMA/RMB%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%25/22/20/20</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%Benteh David%ED3-METE%83%VSLA/303/N1%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/25/23</t>
+  </si>
+  <si>
+    <t>STAT 253%PROBABILITY AND STATISTICS%Awiakye-Marfo George%ED3-CE%223%PB014/PB020/PB201/PB214/PB008/PB208%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%42/42/42/42/28/27</t>
+  </si>
+  <si>
+    <t>CE 255%THEORY OF STRUCTURES%Ampofo James Wiafe%ED2-GEOL%154%VSLA/LT/303/RMA/RMB/304%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/25/25/20/20/24</t>
+  </si>
+  <si>
+    <t>CE 255%THEORY OF STRUCTURES%Ampofo James Wiafe%ED2-CE%260%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2/PB001%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%75/75/50/25/35</t>
+  </si>
+  <si>
+    <t>MSE 451%COMPOSITE MATERIALS%Asare Eric Kwame Anokye%ED4-MSE%64%206/N1/N2%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%24/20/20</t>
+  </si>
+  <si>
+    <t>CE 473%DEVELOPMENT ENGINEERING%Tuffour Yaw Adubofour%ED4-CE%245%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%80/80/55/30</t>
+  </si>
+  <si>
+    <t>CHE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-CHE%120%NAF1/EA/A110/VCR%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30/20</t>
+  </si>
+  <si>
+    <t>CHE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-PCE%56%NEB-FF1%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%56</t>
+  </si>
+  <si>
+    <t>PE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-PE%129%VSLA/LT/303/206/N2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/25/20/14</t>
+  </si>
+  <si>
+    <t>MSE 153%INTRODUCTION TO INFORMATION TECHNOLOGY%Okae James%ED1-MSE%98%304/N1/RMA/RMB%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25/24/24</t>
+  </si>
+  <si>
+    <t>MSE 153%INTRODUCTION TO INFORMATION TECHNOLOGY%Okae James%ED1-METE%72%PB201/PB208%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/27</t>
+  </si>
+  <si>
+    <t>METE 251%METALLURGICAL THERMODYNAMICS%Gikunoo Emmanuel%ED2-METE%59%PB214/PB008%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/19</t>
+  </si>
+  <si>
+    <t>TE 353%RANDOM VARIABLES AND STOCHASTIC PROCESSES%Obour Agyekum Kwame Opuni-Boachie%ED3-TEL%147%PB001/PB020/PB014/PB212%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/12</t>
+  </si>
+  <si>
+    <t>ME 355%STRENGTH OF MATERIALS II%Agyei Agyemang Anthony%ED3-AE%105%NEB-SF/NEB-FF2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%80/23</t>
+  </si>
+  <si>
+    <t>AE 471%FARM STRUCTURES%Bart Plange Ato%ED4-AE%103%NAF1/EA/A110%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%43/30/30</t>
+  </si>
+  <si>
+    <t>GE 451%GEODETIC SURVEYING II%Fosu Collins%ED4-GEOM%93%304/N1/RMA/RMB%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/24/22/22</t>
+  </si>
+  <si>
+    <t>EE 167%OCCUPATIONAL HEALTH AND SAFETY%Asiedu Charlotte%ED1-EE%287%PB001/PB020/PB014/PB201/PB214/PB008/PB208/PB212%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/40/40/26/26/20</t>
+  </si>
+  <si>
+    <t>PE 367%STATISTICS FOR PETROLEUM ENGINEERS%Adjei Stephen%ED3-PE%82%NEB-TF%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%82</t>
+  </si>
+  <si>
+    <t>BME 463%BIOMATERIALS II%Agyapong Dorothy Araba Yakoba%ED4-BME%84%NEB-TF%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%84</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Oppong Tawiah Peter%ED1-TEL%129%VSLA/LT/303/206/N2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/25/20/14</t>
+  </si>
+  <si>
+    <t>GE 263%INFORMATION SCIENCE AND PROGRAMMING%Tienaah Titus%ED2-GEOM%134%NEB-SF/NEB-FF1%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/50</t>
+  </si>
+  <si>
+    <t>ME 255%STRENGTH OF MATERIALS I%Andoh Prince Yaw%ED2-ME%242%Computer Based%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%242</t>
+  </si>
+  <si>
+    <t>ME 255%STRENGTH OF MATERIALS I%Andoh Prince Yaw%ED2-PE%97%Computer Based%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%97</t>
+  </si>
+  <si>
+    <t>ME 255%STRENGTH OF MATERIALS I%Agyei Agyemang Anthony%ED2-AERO%74%NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/24</t>
+  </si>
+  <si>
+    <t>ME 255%STRENGTH OF MATERIALS I%Boahen Samuel%ED2-AE%155%NAF1/EA/A110/ECR/VCR%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/30/30/25/25</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED1-CE%32%PB014%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%32</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED1-GEOL%34%PB020%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%34</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-MSE%13%303%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%13</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-BME%17%PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%17</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTION TO ECONOMICS %Takyi Paul Owusu%ED1-AUTO%88%VSLA/LT/206%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/26/17</t>
+  </si>
+  <si>
+    <t>ECON 151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED2-EE%142%NAF1/EA/A110/ECR/VCR%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/30/30/20/20</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-TEL%30%303%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30</t>
+  </si>
+  <si>
+    <t>ECON 151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED2-COE%36%PB001%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%36</t>
+  </si>
+  <si>
+    <t>ECON151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED3-GEOM%16%PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%16</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED3-PCE%26%PB214%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%26</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTION TO ECONOMICS I%Takyi Paul Owusu%ED3-ME%230%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%85/80/45/20</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED3-CHE%32%PB201%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/12</t>
+  </si>
+  <si>
+    <t>ECON 151%INTRODUCTION TO ECONOMICS I%Takyi Paul Owusu%ED3-AERO%76%VSLA/LT%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/26</t>
+  </si>
+  <si>
+    <t>TE 455%MICROWAVE ENGINEERING%Abdul-Rahman Ahmed%ED4-TEL%142%NEB-TF/NEB-SF%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/62</t>
+  </si>
+  <si>
+    <t>IE 357%PROJECT MANAGEMENT%Asiedu Charlotte%ED3-IND%72%RMA/RMB/206%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%24/24/24</t>
+  </si>
+  <si>
+    <t>CE 451%STRUCTURAL ENGINEERING I%Osei Jack Banahene%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB208/PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/40/40/40/40/30/15</t>
+  </si>
+  <si>
+    <t>COE 281%PROGRAMMING AND PROBLEM SOLIVING%Adjaidoo Theresa-Samuelle Maame Atwemaah%ED2-COE%253%Computer Based%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%253</t>
+  </si>
+  <si>
+    <t>ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Sackey Michael Nii%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%85/85/52/20</t>
+  </si>
+  <si>
+    <t>ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Asante Eric Amoah%ED2-AE%155%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/30/30/25/25</t>
+  </si>
+  <si>
+    <t>MSE 255%ELECTRICAL AND MAGNETIC BEHAVIOUR OF MATERIALS%Dzikunu Perseverance%ED2-MSE%80%NEB-TF/NEB-FF2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%60/20</t>
+  </si>
+  <si>
+    <t>MSE 255%ELECTRICAL AND MAGNETIC BEHAVIOUR OF MATERIALS%Dzikunu Perseverance%ED2-METE%59%NEB-SF%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%59</t>
+  </si>
+  <si>
+    <t>CE 151%ELEMENTARY STRUCTURES%Afrifa Russel Owusu%ED1-GEOL%119%VSLA/LT/303/RMA%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%50/30/20/20</t>
+  </si>
+  <si>
+    <t>PCE 355%FIRE AND SAFETY ENGINEERING%Momade Zsuzsanna Gál%ED3-PCE%51%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%30/21</t>
+  </si>
+  <si>
+    <t>CHE 459%SAFETY AND POLLUTION CONTROL%Ohemeng-Boahen Godfred%ED4-CHE%114%VSLA/LT/303/RMA%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%44/30/20/20</t>
+  </si>
+  <si>
+    <t>GED 267%COMPUTER PROGRAMMING%Kwaw Albert Kwame%ED2-GEOL%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/30/30/25/25</t>
+  </si>
+  <si>
+    <t>EE 387%CLASSICAL CONTROL SYSTEMS%Opoku Daniel%ED3-EE%254%PB001/PB020/PB014/PB201/PB214/PB008%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/45/45/45/45/30</t>
+  </si>
+  <si>
+    <t>MME 353%MARINE ELECTRICAL TECHNOLOGY%Frimpong Emmanuel Asuming%ED3-MARI%40%PB008/PB208%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20</t>
+  </si>
+  <si>
+    <t>GE 171%APPLIED OPTICS%Andam-Akorful Samuel Ato%ED1-GEOM%100%304/N1/RMB/206/N2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%25/25/20/20/10</t>
+  </si>
+  <si>
+    <t>COE 387%CLASSICAL CONTROL SYSTEMS%Klogo Griffith Selorm%ED3-BME%94%304/N1/RMB/206/N2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20/20/20/10</t>
+  </si>
+  <si>
+    <t>COE 387%CLASSICAL CONTROL SYSTEMS%Klogo Griffith Selorm%ED3-COE%276%PB001/PB020/PB014/PB201/PB214/PB208/PB212%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/45/45/45/45/30/21</t>
+  </si>
+  <si>
+    <t>CHE 261%COMPUTER APPLICATIONS FOR ENGINEERS%Bonsu Jude Kwaku%ED2-PCE%59%Computer Based%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%59</t>
+  </si>
+  <si>
+    <t>CHE 261%COMPUTER APPLICATIONS FOR ENGINEERS%Anang Daniel Adjah%ED2-CHE%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/30/30/25/25</t>
+  </si>
+  <si>
+    <t>CE 151%ELEMENTARY STRUCTURES%Afrifa Russel Owusu%ED1-CE%242%PB001/PB020/PB014/PB201/PB214/PB208%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/45/45/20</t>
+  </si>
+  <si>
+    <t>MSE 155%PRINCIPLES OF MATERIALS SCIENCE%Nartey Martinson Addo%ED1-MSE%98%PB208/PB008/PB214%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/30/38</t>
+  </si>
+  <si>
+    <t>ME 365%THERMODYNAMICS  II%Forson Francis Kofi%ED3-AE%105%NAF1/EA/A110/ECR%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/25/20/20</t>
+  </si>
+  <si>
+    <t>ME 365%THERMODYNAMICS  II%Forson Francis Kofi%ED3-ME%230%PB001/PB020/PB014/PB201/PB008/PB212%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/42/43/30/25</t>
+  </si>
+  <si>
+    <t>CE 463%WATER AND WASTE WATER ENGINEERING%Buamah Richard Akwasi%ED4-CE%245%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%85/85/52/23</t>
+  </si>
+  <si>
+    <t>COE 281%PROGRAMMING AND PROBLEM SOLIVING%Adjei Prince Ebenezer%ED2-BME%87%VSLA/LT/RMA%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/21/21</t>
+  </si>
+  <si>
+    <t>TE 251%ANALOG COMMUNICATION SYSTEMS%Affum Emmanuel Ampoma%ED2-TEL%179%VSLA/RMA/303/304/N1/N2/206%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/20/30/22/25/20/17</t>
+  </si>
+  <si>
+    <t>METE 351%PRINCIPLES OF HYDROMETALLURGY%Koomson Bennetta%ED3-METE%83%303/LT/RMB%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/30/23</t>
+  </si>
+  <si>
+    <t>MSE 355%POLYMER PROCESSING%Asare Eric Kwame Anokye%ED3-MSE%89%304/N1/RMB/206%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%25/25/20/20</t>
+  </si>
+  <si>
+    <t>CHE 455%PROCESS CONTROL AND INSTRUMENTATION%Baidoo Martina Francisca%ED4-PCE%62%NEB-TF%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%62</t>
+  </si>
+  <si>
+    <t>PE 357%PETROLEUM PRODUCTION ENGINEERING I%Sarkodie Kwame%ED3-PE%82%NEB-SF%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%82</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Ayetor Godwin Kafui Kwesi%ED2-MARI%37%Computer Based %Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%Computer Based </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Ayetor Godwin Kafui Kwesi%ED2-AUTO%77%Computer Based %Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%Computer Based </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Ayetor Godwin Kafui Kwesi%ED2-IND%80%Computer Based %Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%Computer Based </t>
+  </si>
+  <si>
+    <t>AERO 351%AERODYNAMICS I%Bofah Kwasi Kete%ED3-AERO%76%304/N1/N2/RMA%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%20/20/20/16</t>
+  </si>
+  <si>
+    <t>GED 369%PHOTOGEOLOGY AND REMOTE SENSING%Nuamah Daniel Oduro Boatey%ED3-GEOL%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/30/30/25/25</t>
+  </si>
+  <si>
+    <t>GE 361%IMAGE PROCESSING AND INTERPRETATION%Asare Yaw Mensah %ED3-GEOM%115%NEB-SF/NEB-FF1%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%70/45</t>
+  </si>
+  <si>
+    <t>GED 461%EXPLORATION GEOPHYSICS%Ali Bukari%ED4-GEOL%102%VSLA/LT/303%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%50/26/26</t>
+  </si>
+  <si>
+    <t>CE 259%ENGINEERING GEOLOGY%Acquaah Vincent Kofi Abaka%ED2-CE%260%PB001/PB020/PB014/PB201/PB214/PB208/PB212%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/45/45/40/20/20</t>
+  </si>
+  <si>
+    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Mensah Lena Dzifa%ED4-ME%144%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/30/30/25/15</t>
+  </si>
+  <si>
+    <t>ME 491%ENGINEERING ECONOMICS AND MANAGEMENT%Mensah Lena Dzifa%ED4-EE%224%PB001/PB020/PB014/PB201/PB214%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/45/45/44</t>
+  </si>
+  <si>
+    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Mensah Lena Dzifa%ED4-IND%67%NEB-TF%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%67</t>
+  </si>
+  <si>
+    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Mensah Lena Dzifa%ED4-MSE%64%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/24</t>
+  </si>
+  <si>
+    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Mensah Lena Dzifa%ED4-METE%49%RMB/206%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%24/25</t>
+  </si>
+  <si>
+    <t>MME 491%MARINE ENGINEERING ECONOMY, ACCOUNTING AND MANAGEMENT%Mensah Lena Dzifa%ED4-MARI%23%RMB%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%23</t>
+  </si>
+  <si>
+    <t>AERO 491%AVIATION BUSINESS MANAGEMENT%Takyi Gabriel%ED4-AERO%61%PB008/PB208/PB212%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%20/25/16</t>
+  </si>
+  <si>
+    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Asiedu Charlotte%ED4-AUTO%32%PB008%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%32</t>
+  </si>
+  <si>
+    <t>ME 491%ENGINEERING ECONOMICS AND MANAGEMENT%Mensah Lena Dzifa%ED4-COE%170%NEB-TF/NEB-SF%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%85/85</t>
+  </si>
+  <si>
+    <t>ME 491%ENGINEERING ECONOMICS AND MANAGEMENT%Aikins Stephen Hill Mends%ED4-AE%103%VSLA/LT/303%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%50/26/27</t>
+  </si>
+  <si>
+    <t>ME 491%ENGINEERING ECONOMICS AND MANAGEMENT%Mensah Lena Dzifa%ED4-BME%84%304/N1/N2/RMA%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%25/25/20/14</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Abdul-Rahman Ahmed%ED1-TEL%129%NAF1/EA/A110/VCR%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Acheampong Francisca Adoma%ED1-AUTO%88%N1/N2/206/304%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%22/22/22/22</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Acheampong Francisca Adoma%ED1-MARI%46%N2/RMA%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%23/23</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Affum Emmanuel Ampoma%ED1-ME%223%NEB-TF/NEB-SF/NEB-FF1%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%85/85/55</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Evils Twumasi%ED1-METE%72%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/22</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Ellis Sani Mubarak%ED1-PE%129%NAF1/EA/A110/ECR%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Evils Twumasi%ED1-CHE%120%NEB-SF/NEB-FF2%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%85/35</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Prah II Nicholas Kwesi%ED1-AE%126%VSLA/LT/RMA/RMB%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/30/24/24</t>
+  </si>
+  <si>
+    <t>COE 181%APPLIED ELECTRICITY%Oteng Gyasi Kwame%ED1-COE%261%PB001/PB020/PB014/PB201/PB214/PB008/PB212%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/45/45/45/45/30/6</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Effah Francis Boafo%ED1-EE%287%PB001/PB020/PB014/PB201/PB214/PB008/PB208/PB212%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/45/45/45/45/30/30/2</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Evils Twumasi%ED1-PCE%56%ECR/VCR%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/26</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Obeng Kwakye Kingsford Sarkodie%ED1-IND%81%NEB-TF%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%81</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Oteng Gyasi Kwame%ED1-AERO%70%PB208/PB212%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/40</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Obeng Kwakye Kingsford Sarkodie%ED1-BME%136%VSLA/LT/303/N1%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/30/30/26</t>
+  </si>
+  <si>
+    <t>EE 151%APPLIED ELECTRICITY%Oteng Gyasi Kwame%ED1-MSE%98%303/304/RMB/206%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/25/24/24</t>
+  </si>
+  <si>
+    <t>COE 475%COMPUTER NETWORKING%Akowuah Emmanuel Kofi%ED4-COE%170%Computer Based%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%170</t>
+  </si>
+  <si>
+    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-AERO%74%PB201/PB208/PB212%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/14</t>
+  </si>
+  <si>
+    <t>ME 261%ENGINEERING MECHANICS II: DYNAMICS%Ampofo Joshua%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/80/50/27</t>
+  </si>
+  <si>
+    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-MARI%37%A110/ECR%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/17</t>
+  </si>
+  <si>
+    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-IND%80%VSLA/LT%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%50/30</t>
+  </si>
+  <si>
+    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-AUTO%77%N1/RMA/206/N2%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20/20/17</t>
+  </si>
+  <si>
+    <t>MSE 361%STRESS AND STRAIN ANALYSIS OF RIGID BODIES%Mensah-Darkwa Kwadwo%ED3-MSE%89%NAF1/EA/VCR%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/30/14</t>
+  </si>
+  <si>
+    <t>METE 353%STRENGTH OF MATERIALS%Mensah-Darkwa Kwadwo%ED3-METE%83%303/304/RMA/RMB%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%30/20/20/13</t>
+  </si>
+  <si>
+    <t>IE 367%ETHICS, CONTRACT &amp; PRODUCT LIABILITY LAW%Asiedu Charlotte%ED3-IND%72%PB214/PB008%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%42/30</t>
+  </si>
+  <si>
+    <t>MSE 257%MATERIALS PROCESSING%Agyemang Frank Ofori%ED2-MSE%80%NAF1/EA/VCR%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/20/15</t>
+  </si>
+  <si>
+    <t>PCE 457%CORROSION ENGINEERING%Anang Daniel Adjah%ED4-PCE%62%RMB/206/N1%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20/22</t>
+  </si>
+  <si>
+    <t>AE 351%SOIL AND WATER ENGINEERING%Kyei-Baffour Nicholas%ED3-AE%105%VSLA/LT/303%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%50/28/27</t>
+  </si>
+  <si>
+    <t>TE 271%ANALOG COMMUNICATION SYSTEMS%Ellis Sani Mubarak%ED3-EE%254%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/85/55/29</t>
+  </si>
+  <si>
+    <t>CHE 371%NATURAL GAS PROCESSING TECHNOLOGY%Benjamin Asante%ED3-CHE%50%PB208/PB008%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25</t>
+  </si>
+  <si>
+    <t>TE 453%MOBILE AND WIRELESS COMMUNICATIONS%Agyekum Kwame Agyeman-Prempeh%ED4-TEL%142%PB001/PB020/PB014/PB212%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/40/42/15</t>
+  </si>
+  <si>
+    <t>ME 361%DYNAMICS OF MACHINERY%Ampofo Joshua%ED3-MARI%40%N2/206%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20</t>
+  </si>
+  <si>
+    <t>ME 361%DYNAMICS OF MACHINERY%Ampofo Joshua%ED3-AUTO%47%A110/ECR%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/22</t>
+  </si>
+  <si>
+    <t>ME 361%DYNAMICS OF MACHINERY%Sackey Samuel Mensah%ED3-ME%230%PB001/PB020/PB014/PB201/PB214/PB212%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/40/40/40/20</t>
+  </si>
+  <si>
+    <t>GE 371%SURVEY ADJUSTMENT I%Fosu Collins%ED3-GEOM%115%Computer Based%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%115</t>
+  </si>
+  <si>
+    <t>GE 271%ENGINEERING SURVEYING I%Arko-Adjei Anthony%ED2-GEOM%134%PB214/PB212/PB208/PB008%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/29/30/30</t>
+  </si>
+  <si>
+    <t>CHE 251%CHEMICAL PROCESS CALCULATIONS I%Rockson Mizpah Ama Dziedzorm%ED2-CHE%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/30/30/25/25</t>
+  </si>
+  <si>
+    <t>CHE 251%CHEMICAL PROCESS CALCULATIONS I%Ohemeng-Boahen Godfred%ED2-PCE%59%PB208/PB008%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30/29</t>
+  </si>
+  <si>
+    <t>ARC 155%CLIMATE AND ARCHITECTURE%Amos-Abanyie Samuel%ED1-CE%74%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/24</t>
+  </si>
+  <si>
+    <t>PE 359%RESERVOIR PETROPHYSICS%Erzuah Samuel%ED3-PE%82%NEB-SF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%82</t>
+  </si>
+  <si>
+    <t>CE 479%ENGINEERING AND ENVIRONMENTAL GEOPHYSICS%Owusu-Nimo Frederick%ED4-CE%245%VSLA/LT/RMA/RMB/303/304/206/N1/N2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/25/24/24/30/21/24/25/22</t>
+  </si>
+  <si>
+    <t>PE 451%PETROLEUM ECONOMICS%Quaye Jonathan Atuquaye%ED4-PE%103%NEB-SF/NEB-FF2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/23</t>
+  </si>
+  <si>
+    <t>PE 255%FLUID MECHANICS%Adjei Stephen%ED2-PE%97%NEB-TF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%97</t>
+  </si>
+  <si>
+    <t>TE 253%DIGITAL SYSTEMS%Obour Agyekum Kwame Opuni-Boachie%ED2-TEL%179%PB001/PB020/PB014/PB201%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45</t>
+  </si>
+  <si>
+    <t>TE 355%SIGNALS AND SYSTEMS%Agyekum Kwame Agyeman-Prempeh%ED3-TEL%147%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/30/30/21/21</t>
+  </si>
+  <si>
+    <t>PCE 357%ORGANIC AND PETROCHEMICAL SYNTHESIS%Mensah Mary%ED3-PCE%51%NEB-TF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%51</t>
+  </si>
+  <si>
+    <t>CE 353%REINFORCED CONCRETE DESIGN%Owusu Twumasi Jones%ED3-CE%223%PB001/PB020/PB014/PB201/PB214/PB212%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%41/42/40/40/40/20</t>
+  </si>
+  <si>
+    <t>GE 161%BASIC SURVEY PRINCIPLES I%Ayer John Wise Divine%ED1-GEOM%100%VSLA/LT/RMA/RMB%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/20/20/20</t>
+  </si>
+  <si>
+    <t>GE 475%RESEARCH METHODS%Duker Alfred Alan%ED4-GEOM%93%303/304/206/N1/N2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%25/18/18/18/14</t>
+  </si>
+  <si>
+    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sackey Michael Nii%ED1-AERO%70%NAF1/A110%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%42/28</t>
+  </si>
+  <si>
+    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sackey Michael Nii%ED1-ME%223%VSLA/LT/303/304/N1/RMA/RMB/206/N2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%44/26/26/22/22/21/21/21/20</t>
+  </si>
+  <si>
+    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sekyere Charles Kofi Kafui%ED1-MARI%46%A110/VCR%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%23/23</t>
+  </si>
+  <si>
+    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sekyere Charles Kofi Kafui%ED1-IND%81%303/304/206/RMB%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%25/20/20/20</t>
+  </si>
+  <si>
+    <t>EE 271%SEMICONDUCTOR DEVICES%Sekyere Yaw Opoku Mensah%ED2-EE%340%PB001/PB014/PB020/PB201/PB214/PB008/PB208/PB212/EA%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/45/45/45/45/30/30/25/30</t>
+  </si>
+  <si>
+    <t>COE 271%SEMICONDUCTOR DEVICES%Kommey Benjamin%ED2-BME%87%VSLA/LT/RMA%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/27/21</t>
+  </si>
+  <si>
+    <t>COE 271%SEMICONDUCTOR DEVICES%Kommey Benjamin%ED2-COE%253%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%85/85/55/28</t>
+  </si>
+  <si>
+    <t>EE 371%LINEAR ELECTRONIC CIRCUITS%Sekyere Yaw Opoku Mensah%ED3-EE%254%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%85/85/55/29</t>
+  </si>
+  <si>
+    <t>IE 365%ENGINEERING WORK STUDY%Takyi Gabriel%ED3-IND%72%NAF1/EA%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%44/28</t>
+  </si>
+  <si>
+    <t>EE 153%ELECTRICAL ENGINEERING TECHNOLOGY WITH MATLAB%Prah II Nicholas Kwesi%ED1-EE%287%PB001/PB014/PB020/PB201/PB214/PB208/PB008/PB212%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%42/42/42/42/42/30/28/20</t>
+  </si>
+  <si>
+    <t>GED 151%BASIC GEOLOGY%Gawu Simon Kafui Yawo%ED1-GEOL%119%VSLA/RMA/303/N2%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/30/24/15</t>
+  </si>
+  <si>
+    <t>PE 253%BASIC GEOLOGY%Quaye Jonathan Atuquaye%ED2-PE%97%LT/304/RMA/206%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/25/24/18</t>
+  </si>
+  <si>
+    <t>AE 373%MACHINE DESIGN I%Aveyire Joseph%ED3-AE%105%VSLA/304/RMB/N2%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/25/24/6</t>
+  </si>
+  <si>
+    <t>PE 155%INTRODUCTION TO INFORMATION TECHNOLOGY%Sokama-Neuyam Yen Adams%ED1-PE%129%PB020/PB201/PB008/PB212%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/30/9</t>
+  </si>
+  <si>
+    <t>CHE 253%CHEMICAL ENGINEERING THERMODYNAMICS I%Bonsu Jude Kwaku%ED2-CHE%154%PB001/PB014/PB214/PB208%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/19</t>
+  </si>
+  <si>
+    <t>CHE 253%CHEMICAL ENGINEERING THERMODYNAMICS I%Dogbe Eunice Sefakor Aku%ED2-PCE%59%NAF1/A110%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%39/20</t>
+  </si>
+  <si>
+    <t>AERO 391%AEROSPACE INDUSTRY AND ENGINEERING%K. K. Bofah%ED3-AERO%76%NEB-TF%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/25/21</t>
+  </si>
+  <si>
+    <t>MSE 253%MECHANICAL BEHAVIOUR OF MATERIALS%Kwofie Samuel%ED2-MSE%80%LT/N1/RMB%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/25/25</t>
+  </si>
+  <si>
+    <t>MSE 253%MECHANICAL BEHAVIOUR OF MATERIALS%Kwofie Samuel%ED2-METE%59%303/N1/206%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%20/20/19</t>
+  </si>
+  <si>
+    <t>GE 251%PRINCIPLES OF PHOTOGRAMMETRY%Ahorsu Harriet Atsufui%ED2-GEOM%134%PB020/PB201/PB008/PB212%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/30/14</t>
+  </si>
+  <si>
+    <t>CE 153%ENGINEERING PRACTICE AND TECHNOLOGY%Acquaah Vincent Kofi Abaka%ED1-CE%242%NEB-SF/NEB-FF1/NEB-FF2/NAF1/EA/VCR%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%80/50/20/40/30/25</t>
+  </si>
+  <si>
+    <t>CE 251%STRENGTH OF MATERIALS%Amponsah Evans%ED2-CE%260%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%85/85/55/35</t>
+  </si>
+  <si>
+    <t>CE 251%STRENGTH OF MATERIALS%Kankam Charles Kwame%ED2-GEOL%154%PB001/PB014/PB214/PB208%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/19</t>
+  </si>
+  <si>
+    <t>CHE 363%POLYMER TECHNOLOGY%Boakye Patrick%ED3-CHE%36%ECR/VCR%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%25/11</t>
+  </si>
+  <si>
+    <t>CHE 363%POLYMER TECHNOLOGY%Boakye Patrick%ED3-PCE%51%A110/EA%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%31/20</t>
+  </si>
+  <si>
+    <t>EE 287%CIRCUIT THEORY%Gadze James Dzisi%ED2-TEL%179%PB001/PB014/PB214/PB208/PB212%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/45/38/9</t>
+  </si>
+  <si>
+    <t>COE 475%COMPUTER NETWORKING%Adrah Charles Mawutor%ED4-EE%224%PB001/PB020/PB014/PB201/PB008/PB212%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/45/45/30/14</t>
+  </si>
+  <si>
+    <t>TE 465%DIGITAL INTEGRATED CIRCUITS%Affum Emmanuel Ampoma%ED4-TEL%142%PB020/PB201/PB008/PB208%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/30/22</t>
+  </si>
+  <si>
+    <t>IE 457%ADVANCED MANUFACTURING TECHNOLOGY II%Takyi Gabriel%ED4-IND%67%PB214/PB212%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/22</t>
+  </si>
+  <si>
+    <t>GE 381%ENGINEERING SURVEYING I%Obeng Kwame%ED3-CE%223%NEB-SF/NEB-TF/NEB-FF1%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%85/85/53</t>
+  </si>
+  <si>
+    <t>MSE 457%METALWORKING PROCESSES%Kwofie Samuel%ED4-MSE%64%304/RMA/N2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%25/24/15</t>
+  </si>
+  <si>
+    <t>MSE 457%METAL FORMING PROCESSES%Kwofie Samuel%ED4-METE%49%A110/ECR%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%30/19</t>
+  </si>
+  <si>
+    <t>CHE 463%ELECTROCHEMICAL TECHNOLOGY%Anang Daniel Adjah%ED4-PCE%18%A110%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%18</t>
+  </si>
+  <si>
+    <t>CHE 463%ELECTROCHEMICAL TECHNOLOGY%Anang Daniel Adjah%ED4-CHE%40%NAF1%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40</t>
+  </si>
+  <si>
+    <t>CE 477%GEOTECHNICAL ENGINEERING I%Ayeh Felix Jojo Fianko%ED4-CE%245%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%80/80/55/30</t>
+  </si>
+  <si>
+    <t>CE 477%GEOTECHNICAL ENGINEERING I%Ampadu Samuel Innocent Kofi%ED4-GEOL%102%LT/303/RMA/206%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%30/30/24/18</t>
+  </si>
+  <si>
+    <t>AE 451%IRRIGATION AND DRAINAGE%Agodzo Sampson Kwaku%ED4-AE%103%VSLA/N1/RMB/N2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/25/24/9</t>
+  </si>
+  <si>
+    <t>PE 361%RESERVOIR ENGINEERING II%Adenutsi Caspar Daniel%ED3-PE%82%303/N1/206%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%30/25/27</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Amoabeng Kofi Owura%ED1-BME%136%VSLA/LT/304/RMB/N2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%50/30/25/24/7</t>
+  </si>
+  <si>
+    <t>MME 473%MARINE MACHINERY SYSTEM DESIGN%Sackey Michael Nii%ED4-MARI%23%ECR%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%23</t>
+  </si>
+  <si>
+    <t>COE 253%DISCRETE STRUCTURES%Kwabi Prince Amponsah%ED2-COE%253%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%85/85/53/30</t>
+  </si>
+  <si>
+    <t>ME 451%BEHAVIOUR OF REAL FLUIDS%Opoku Richard%ED4-ME%144%NAF1/EA/A110/VCR/ECR%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/30/30/25/20</t>
+  </si>
+  <si>
+    <t>ME 451%BEHAVIOUR OF REAL FLUIDS%Opoku Richard%ED4-AERO%61%RMA/RMB/206%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%21/20/20</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-MSE%98%PB201/PB208/PB212%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%43/30/25</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-TEL%129%PB001/PB014/PB020%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%43/43/43</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-MARI%46%N2/206%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%23/23</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-ME%223%VSLA/LT/303/304/RMA/RMB/N1/N2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/24/24/24/24/23</t>
+  </si>
+  <si>
+    <t>SES 171%FUNDAMENTALS OF ACQUATIC SKILLS%Afrifa Daniel%ED2-MARI%40%PB214%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40</t>
+  </si>
+  <si>
+    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-ME%242%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%81/81/50/30</t>
+  </si>
+  <si>
+    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-AERO%74%NAF1/A110%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%44/30</t>
+  </si>
+  <si>
+    <t>ME 251%FLUID MECHANICS I%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-AE%155%VSLA/LT/303/N1/304%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25/24</t>
+  </si>
+  <si>
+    <t>AME 371%LAND VEHICLE DESIGN%Ayetor Godwin Kafui Kwesi%ED3-AUTO%47%VCR/ECR%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%24/23</t>
+  </si>
+  <si>
+    <t>EE 261%DC MACHINES%Effah Francis Boafo%ED2-EE%340%PB001/PB014/PB020/PB201/PB214/PB008/PB208/PB212/EA%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/45/45/45/45/30/30/25/30</t>
+  </si>
+  <si>
+    <t>IE 363%PROCESS PLANNING SYSTEMS%Sackey Samuel Mensah%ED3-IND%72%ECR/VCR/A110%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25/22</t>
+  </si>
+  <si>
+    <t>MSE 363%MATERIALS CHARACTERIZATION TECHNIQUE%Arthur Emmanuel Kwesi%ED3-METE%83%RMA/RMB/N1/206%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%21/21/21/20</t>
+  </si>
+  <si>
+    <t>MSE 363%MATERIALS CHARACTERIZATION TECHNIQUE%Arthur Emmanuel Kwesi%ED3-MSE%89%NEB-TF/NEB-FF2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%64/25</t>
+  </si>
+  <si>
+    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-COE%276%PB001/PB020/PB014/PB201/PB214/PB008/PB212%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/45/45/30/21</t>
+  </si>
+  <si>
+    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-BME%94%NAF1/EA/VCR%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/24</t>
+  </si>
+  <si>
+    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-EE%254%PB001/PB020/PB014/PB201/PB214/PB208%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/45/45/29</t>
+  </si>
+  <si>
+    <t>CHE 351%MASS TRANSFER PROCESSES%Ankudey Emmanuel Godwin%ED3-CHE%100%NAF1/EA/A110%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Boahen Samuel%ED1-GEOL%119%VSLA/LT/303/304%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/25/24</t>
+  </si>
+  <si>
+    <t>BME 265%BIOLOGICAL TRANSPORT PHENOMENA%Odame Prince%ED2-BME%87%RMA/RMB/N1/N2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%22/22/22/21</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Boahen Samuel%ED1-PCE%56%PB208/PB008%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%28/28</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Asante Eric Amoah%ED1-CHE%120%VSLA/LT/303/304%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30/20</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Aveyire Joseph%ED1-CE%242%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/85/50/22</t>
+  </si>
+  <si>
+    <t>ME 159%TECHNICAL DRAWING%Aveyire Joseph%ED1-AE%126%NEB-SF/NEB-FF1%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%75/51</t>
+  </si>
+  <si>
+    <t>CE 359%SOIL MECHANICS%Charkley Frederick Nai%ED3-CE%223%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%75/75/50/23</t>
+  </si>
+  <si>
+    <t>GED 379%SOIL MECHANICS%Amenuvor Andrew Cudzo%ED3-GEOL%154%VSLA/LT/303/304/206%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%49/30/30/25/20</t>
+  </si>
+  <si>
+    <t>PE 259%SURVIVAL SWIMMING TECHNIQUES%Gyamfi Isaac%ED2-PE%97%VSLA/LT/303/304/206%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/25/20/12</t>
+  </si>
+  <si>
+    <t>PCE 451%CATALYSIS%Baidoo Martina Francisca%ED4-PCE%62%N1/RMA/RMB%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%22/20/20</t>
+  </si>
+  <si>
+    <t>ME 373%MACHINE ELEMENTS DESIGN I%Davis Francis%ED3-ME%230%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/80/50/20</t>
+  </si>
+  <si>
+    <t>GE 351%STEREO PHOTOGRAMMETRY%Tienaah Titus%ED3-GEOM%115%NAF1/EA/A110/VCR%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/30/30/15</t>
+  </si>
+  <si>
+    <t>ME 161%BASIC MECHANICS%Tay Godwin Fabiola Kwaku%ED1-COE%261%PB001/PB020/PB014/PB201/PB214/PB208/PB212%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%42/42/42/42/42/30/21</t>
+  </si>
+  <si>
+    <t>MME 365%ENGINEERING THERMODYNAMICS%Amoabeng Kofi Owura%ED3-MARI%40%ECR/VCR%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/20</t>
+  </si>
+  <si>
+    <t>AME 485%AUTOMATIC POWER TRAIN%Abu Frimpong Solomon%ED4-AUTO%32%RMA/RMB%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%16/16</t>
+  </si>
+  <si>
+    <t>CE 461%ENG ECONOMY AND ENTERPRENEURSHIP DEVELOPMENT%Appiah-Effah Eugene%ED4-GEOM%93%NAF1/EA/A110%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/25/28</t>
+  </si>
+  <si>
+    <t>CE 461%ENGINEERING ECONOMY AND ENTERPRENEURSHIP%Appiah-Effah Eugene%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB212%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45/45/20</t>
+  </si>
+  <si>
+    <t>ME 455%FINITE ELEMENT METHODS%Andoh Prince Yaw%ED4-ME%144%Computer Based%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%144</t>
+  </si>
+  <si>
+    <t>GE 151%CARTOGRAPHY I%Quaye-Ballard Jonathan Arthur%ED1-GEOM%100%PB008/PB208/PB214/PB212%Monday, 23 February 2026%Session, 1 (8:15AM - 9:15 AM)%30/30/20/20</t>
+  </si>
+  <si>
+    <t>GED 253%PHYSICAL GEOLOGY%Mensah Emmanuel%ED2-GEOL%154%PB014/PB001/PB020/PB008%Monday, 23 February 2026%Session, 1 (8:15AM - 9:15 AM)%40/44/40/30</t>
+  </si>
+  <si>
+    <t>CHE 255%FLUID TRANSPORT%Dogbe Eunice Sefakor Aku%ED2-PCE%59%PB214/PB201%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%30/29</t>
+  </si>
+  <si>
+    <t>GED 251%MINERALOGY%Wilson Matthew Coffie%ED2-GEOL%154%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%80/50/24</t>
+  </si>
+  <si>
     <t>MATH 151%ALGEBRA%Barnes Benedict%ED1-PCE%56%PB008/PB208%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/26</t>
-  </si>
-  <si>
-    <t>MATH 151%ALGEBRA%Adu-Ansah Lawton%ED1-TEL%129%VSLA/LT/304/RMA%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/30/25/24</t>
-  </si>
-  <si>
-    <t>MATH 151%ALGEBRA%Azure Isaac%ED1-AUTO%88%RMB/303/N1/N2%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%22/22/22/22</t>
-  </si>
-  <si>
-    <t>MATH 151%ALGEBRA%Ayekple Yao Elikem%ED1-EE%287%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2/NAF1%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%80/85/55/30/37</t>
-  </si>
-  <si>
-    <t>MATH 151%ALGEBRA%Azure Isaac%ED1-GEOM%100%RMB/303/N1/N2%Tuesday, 24 February 2026%Session, 2 (10:00 AM - 11:00 AM)%22/30/24/24</t>
-  </si>
-  <si>
-    <t>TE 357%OPTICAL COMMUNICATION%Gadze James Dzisi%ED3-TEL%147%PB020/PB201/PB214/PB212%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/40/40/25</t>
-  </si>
-  <si>
-    <t>IE 355%DISCRETE EVENT SIMULATION%Takyi Gabriel%ED3-IND%72%VSLA/303%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%44/28</t>
-  </si>
-  <si>
-    <t>AE 457%CROP PROCESSING%Darko Joseph Ofei %ED4-AE%103%VSLA/LT/RMA/RMB%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/25/20/18</t>
-  </si>
-  <si>
-    <t>GED 459%EXPLORATION GEOCHEMISTRY%Gawu Simon Kafui Yawo%ED4-GEOL%102%LT/N1/RMA/RMB/N2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%22/22/20/20/20</t>
-  </si>
-  <si>
-    <t>CE 467%HIGHWAY ENGINEERING II%Tuffour Yaw Adubofour%ED4-CE%245%PB001/PB014/PB201/PB214/PB208/PB008/PB212%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%42/42/42/42/30/28/20</t>
-  </si>
-  <si>
-    <t>COE 485%COMPUTER ARCHITECTURE%Boateng Kwame Osei%ED4-COE%170%PB001/PB014/PB020/PB208/PB008%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/40/40/25/25</t>
-  </si>
-  <si>
-    <t>TE 481%WIRELESS DATA COMMUNICATION NETWORK%Opare Kwasi Adu-Boahen%ED4-EE%224%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%75/75/50/24</t>
-  </si>
-  <si>
-    <t>IE 459%RISK ANALYSIS%Asiedu Charlotte%ED4-IND%67%NAF1/EA%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%40/27</t>
-  </si>
-  <si>
-    <t>CE 355%HYDROLOGY%Adjei Kwaku Amaning%ED3-CE%223%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%75/75/50/23</t>
-  </si>
-  <si>
-    <t>PCE 455%POLLUTION CONTROL IN PETROCHEMICAL INDUSTRY%Kwao-Boateng Emmanuela%ED4-PCE%62%303/206/304%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%22/20/20</t>
-  </si>
-  <si>
-    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-MARI%23%ECR%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%23</t>
-  </si>
-  <si>
-    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-AUTO%32%N1/N2%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%16/16</t>
-  </si>
-  <si>
-    <t>ME 453%HYDRAULICS AND PNEUMATICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED4-ME%144%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 3 ( 11:45 AM - 12:45 PM)%45/30/30/20/20</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Boateng Maxwell Akwasi%ED2-MARI%37%206/RMB%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%20/17</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Boateng Maxwell Akwasi%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%80/80/55/27</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-TEL%179%VSLA/LT/303/N1/N2/RMA%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/30/30/25/24/20</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-GEOL%154%VSLA/303/N1/RMA/RMB/304%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/25/25/20/20/20</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-COE%253%PB001/PB014/PB020/PB201/PB214/PB208/PB212%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/40/40/40/40/28/25</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-IND%80%EA/A110/VCR%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/20/20</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-AE%155%NEB-TF/NEB-SF%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%78/77</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-CE%260%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%42/42/42/42/42/25/25</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Wireko Fredrick Asenso%ED2-AERO%74%NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/24</t>
-  </si>
-  <si>
-    <t>MATH 251%DIFFERENTIAL EQUATIONS%Barnes Benedict%ED2-GEOM%134%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/25/25/20/20</t>
-  </si>
-  <si>
-    <t>AERO 473%AEROSPACE VEHICLE DESIGN%Oppong David Kofi%ED4-AERO%61%NAF1/ECR%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/21</t>
-  </si>
-  <si>
-    <t>CHE 357%EXPERIMENTAL DATA ANALYSIS%Kwao-Boateng Emmanuela%ED3-PCE%51%PB008/PB212%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/21</t>
-  </si>
-  <si>
-    <t>CHE 357%EXPERIMENTAL DATA ANALYSIS%Rockson Mizpah Ama Dziedzorm%ED3-CHE%100%LT/206/N2/304%Tuesday, 24 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/25/24/24</t>
-  </si>
-  <si>
-    <t>CE 155%ENVIRONMENTAL STUDIES%Appiah-Brempong Miriam%ED1-AERO%70%PB208/PB008/PB212%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25/20</t>
-  </si>
-  <si>
-    <t>CE 155%ENVIRONMENTAL STUDIES%Buamah Richard Akwasi%ED1-AE%126%VSLA/LT/303/304%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/30/30/21</t>
-  </si>
-  <si>
-    <t>CE 155%ENVIRONMENTAL STUDIES%Essandoh Helen Michelle Korkor%ED1-COE%261%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%42/42/42/42/42/28/25</t>
-  </si>
-  <si>
-    <t>CE 155%ENVIRONMENTAL STUDIES%Appiah-Brempong Miriam%ED1-IND%81%NEB-TF%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%81</t>
-  </si>
-  <si>
-    <t>CE 155%ENVIRONMENTAL STUDIES%Buamah Richard Akwasi%ED1-TEL%129%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30/22/20</t>
-  </si>
-  <si>
-    <t>CE 155%ENVIRONMENTAL STUDIES%Awuah Esi%ED1-ME%223%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%75/75/55/20</t>
-  </si>
-  <si>
-    <t>CHE 151%INORGANIC CHEMISTRY FOR ENGINEERS%Opoku Francis%ED1-CHE%120%PB001/PB014/PB020%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/40/40</t>
-  </si>
-  <si>
-    <t>CHE 151%INORGANIC CHEMISTRY FOR ENGINEERS%Opoku Francis%ED1-PCE%56%EA/A110%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%28/28</t>
-  </si>
-  <si>
-    <t>PE 151%INORGANIC CHEMISTRY FOR ENGINEERS%Opoku Francis%ED1-PE%129%VSLA/LT/303/N1%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/30/30/25</t>
-  </si>
-  <si>
-    <t>METE 453%METALLURGICAL FAILURE ANALYSIS AND NDTs%Arthur Emmanuel Kwesi%ED4-METE%49%206/304%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/24</t>
-  </si>
-  <si>
-    <t>MSE 455%FAILURE ANALYSIS AND NON-DESTRUCTIVE TESTING%Arthur Emmanuel Kwesi%ED4-MSE%64%RMA/RMB/N2%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%22/22/20</t>
-  </si>
-  <si>
-    <t>MSE 351%ENGINEERING CERAMICS%Andrews Anthony%ED3-MSE%89%NAF1/VCR/ECR%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/25/24</t>
-  </si>
-  <si>
-    <t>GED 351%PETROLOGY%Foli Gordon%ED3-GEOL%154%NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%80/50/30</t>
-  </si>
-  <si>
-    <t>GE 463%LAND AND GEOGRAPHIC INFORMATION SYSTEM I%Forkuo Eric Kwabena%ED4-GEOM%93%PB201/PB214/PB212%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/40/13</t>
-  </si>
-  <si>
-    <t>MME 373%DESIGN OF MARINE MACHINE ELEMENTS%Andoh Prince Yaw%ED3-MARI%40%Computer Based%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40</t>
-  </si>
-  <si>
-    <t>AME 373%DESIGN OF AUTO MECHANICAL SYSTEMS%Andoh Prince Yaw%ED3-AUTO%47%Computer Based%Tuesday, 24 February 2026%Session, 5 (3:15 PM - 4:15 PM)%47</t>
-  </si>
-  <si>
-    <t>PCE 253%INTRODUCTION TO PETROCHEMICAL INDUSTRIES%Baidoo Martina Francisca%ED2-PCE%59%NEB-TF%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%59</t>
-  </si>
-  <si>
-    <t>CHE 259%CHEMICAL PROCESS INDUSTRIES%Afotey Benjamin%ED2-CHE%154%NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/50/24</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Adam Faisal Wahib%ED1-GEOL%119%NAF1/EA/A110/ECR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/27/27/20</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Opoku Richard%ED1-CE%242%VSLA/LT/303/304/RMA/RMB/206/N1/N2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/30/30/25/24/24/20/20/20</t>
-  </si>
-  <si>
-    <t>CE 367%HIGHWAY AND TRANSPORTATION ENGINEERING I%Ababio-Donkor Augustus%ED3-GEOM%115%VSLA/LT/303/304%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%43/26/26/20</t>
-  </si>
-  <si>
-    <t>EE 365%ELECTRICAL SERVICES DESIGN%Kwegyir Daniel%ED3-EE%254%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/40/40/40/40/30/24</t>
-  </si>
-  <si>
-    <t>CE 475%SYSTEMS ENGINEERING I%Donkor Emmanuel Amponsah%ED4-CE%245%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/80/55/30</t>
-  </si>
-  <si>
-    <t>TE 385%SIGNALS AND SYSTEMS%Yeboah-Akowuah Bright%ED3-COE%276%PB001/PB014/PB020/PB201/PB214/PB008/PB212%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45/45/30/21</t>
-  </si>
-  <si>
-    <t>TE 385%SIGNALS AND SYSTEMS%Yeboah-Akowuah Bright%ED3-BME%94%N1/N2/RMA/RMB%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%25/24/23/22</t>
-  </si>
-  <si>
-    <t>TE 463%AVIATION COMMUNICATION%Obeng Kwakye Kingsford Sarkodie%ED4-TEL%142%NAF1/EA/A110/VCR/ECR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/30/30/22/20</t>
-  </si>
-  <si>
-    <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-CHE%39%206/VCR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%24/15</t>
-  </si>
-  <si>
-    <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-PE%3%ECR%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%3</t>
-  </si>
-  <si>
-    <t>PCE 461%FUEL AND COMBUSTION TECHNOLOGY%Ohemeng-Boahen Godfred%ED4-PCE%45%PB208/PB212%Tuesday, 24 February 2026%Session, 6 (5:00 PM - 6:00 PM)%25/20</t>
-  </si>
-  <si>
-    <t>ME 281%ENGINEERING MATERIALS I%Amoabeng Kofi Owura%ED2-AERO%74%A110/EA/VCR%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%28/28/18</t>
-  </si>
-  <si>
-    <t>ME 281%ENGINEERING MATERIALS I%Amoabeng Kofi Owura%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%80/80/55/27</t>
-  </si>
-  <si>
-    <t>AE 153%AGRIC. METEOROLOGY AND CLIMATOLOGY%Bessah Enoch%ED1-AE%126%NEB-SF/NEB-FF1%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%75/51</t>
-  </si>
-  <si>
-    <t>GED 365%GEOLOGICAL FIELD MAPPPING%Brako Blestmond Afrifa%ED3-GEOL%154%VSLA/LT/303/RMA/RMB/304%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/28/28/20/20/18</t>
-  </si>
-  <si>
-    <t>AME 455%VEHICLE AIR-CONDITIONING AND REFRIGERATION%Sekyere Charles Kofi Kafui%ED4-AUTO%32%N1/N2%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%16/16</t>
-  </si>
-  <si>
-    <t>SOC 255%INTRODDUCTION TO RURAL SOCIOLOGY%Boateng Kwabena%ED2-METE%59%N1/N2/206%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20/19</t>
-  </si>
-  <si>
-    <t>SOC 255%INTRODUCTION TO RURAL SOCIOLOGY%Boateng Kwabena%ED3-METE%83%NAF1/VCR/ECR%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/22/22</t>
-  </si>
-  <si>
-    <t>MME 465%MARINE AIR CONDITIONING AND REFRIGERATION%Sekyere Charles Kofi Kafui%ED4-MARI%23%206%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%23</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Dzebre Denis Edem Kwame%ED1-GEOM%100%NEB-TF/NEB-FF2%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%75/25</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Dzebre Denis Edem Kwame%ED1-EE%287%PB001/PB014/PB020/PB201/PB214/PB008/PB208/PB212%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%42/42/42/42/42/30/28/20</t>
-  </si>
-  <si>
-    <t>ME 465%AIR CONDITIONING AND REFRIGERATION%Sekyere Charles Kofi Kafui%ED4-AERO%61%NAF1/ECR%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/21</t>
-  </si>
-  <si>
-    <t>ME 465%AIR CONDITIONING AND REFRIGERATION%Sekyere Charles Kofi Kafui%ED4-ME%144%PB001/PB014/PB020/PB008%Wednesday, 25 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/40/40/25</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Darko Jeel Pharis%ED3-CHE%64%303/206/304%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%24/20/20</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED1-CE%136%PB201/PB214/PB208/PB212%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/40/30/26</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED1-GEOL%80%RMB/N1/N2/304%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%20/20/20/20</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED2-BME%42%NAF1%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%42</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED2-COE%146%PB001/PB014/PB020/PB008%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/40/40/27</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED2-EE%174%VSLA/LT/303/N1/RMA/RMB%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/30/30/24/24/24</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Ocloo Alexander%ED2-MSE%53%NEB-FF1%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%53</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Ocloo Alexander%ED2-TEL%104%NEB-SF/NEB-FF2%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%80/24</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Osei-Danso Harriet Efua%ED3-GEOM%60%A110/EA%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/30</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Boakye-Agyeman Candy%ED1-MARI%46%VCR/ECR%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%23/23</t>
-  </si>
-  <si>
-    <t>FC 181%FRENCH FOR COMMUNICATION PURPOSES I%Darko Jeel Pharis%ED3-PCE%22%PB208%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%22</t>
-  </si>
-  <si>
-    <t>METE 151%INTRODUCTION TO METALLURGICAL ENGINEERING%Koomson Bennetta%ED1-METE%72%NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%47/25</t>
-  </si>
-  <si>
-    <t>AERO 157%INTRODUCTION TO AVIATION TECHNOLOGY%Oppong David Kofi%ED1-AERO%70%NEB-TF%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%70</t>
-  </si>
-  <si>
-    <t>CHEM 151%GENERAL CHEMISTRY%Sarpong Lilian%ED1-BME%136%NAF1/EA/A110/VCR/ECR%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/28/28/20/20</t>
-  </si>
-  <si>
-    <t>EE 371%MICROELECTRONIC CIRCUITS%Acheampong Francisca Adoma%ED3-TEL%147%NEB-SF/NEB-TF%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%74/73</t>
-  </si>
-  <si>
-    <t>COE 371%LINEAR ELECTRONIC CIRCUITS%Agbemenu Andrew Selasi%ED3-COE%276%PB001/PB014/PB020/PB201/PB214/PB008/PB212%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/45/45/30/21</t>
-  </si>
-  <si>
-    <t>COE 371%LINEAR ELECTRONIC CIRCUITS%Agbemenu Andrew Selasi%ED3-BME%94%VSLA/LT/RMA%Wednesday, 25 February 2026%Session, 2 (10:00 AM - 11:00 AM)%42/28/24</t>
-  </si>
-  <si>
-    <t>CHE 257%ANALYTICAL CHEMISTRY FOR CHEMICAL ENGINEERS%Boakye Patrick%ED2-CHE%154%NEB-TF/NEB-SF%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%77/77</t>
-  </si>
-  <si>
-    <t>CHE 257%ANALYTICAL CHEMISTRY FOR CHEMICAL ENGINEERS%Boakye Patrick%ED2-PCE%59%A110/EA/VCR%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%20/20/19</t>
-  </si>
-  <si>
-    <t>ME 281%ENGINEERING MATERIALS I%Boahen Samuel%ED2-AUTO%77%NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%50/27</t>
-  </si>
-  <si>
-    <t>MME 281%MARINE ENGINEERING MATERIALS%Boahen Samuel%ED2-MARI%37%PB208/PB212%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%20/17</t>
-  </si>
-  <si>
-    <t>ME 281%ENGINEERING MATERIALS I%Boahen Samuel%ED2-IND%80%PB001/PB014%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/40</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sekyere Charles Kofi Kafui%ED1-AUTO%88%VSLA/303/304%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/30/18</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sekyere Charles Kofi Kafui%ED1-IND%81%NEB-SF%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%81</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Afriyie Nyarko Frank Kwabena%ED1-COE%261%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%42/42/42/42/42/26/25</t>
-  </si>
-  <si>
-    <t>PE 455%RESERVOIR SIMULATION%Ampomah William%ED4-PE%103%NEB-TF/NEB-FF2%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%78/25</t>
-  </si>
-  <si>
-    <t>GED 465%ENGINEERING GEOLOGICAL INVESTIGATIONS%Ali Bukari%ED4-GEOL%102%PB201/PB214/PB208%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/40/23</t>
-  </si>
-  <si>
-    <t>GE 281%BASIC PHYSICAL GEODESY%Dadzie Isaac%ED2-GEOM%134%VSLA/LT/303/RMA/RMB%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/27/27/22/22</t>
-  </si>
-  <si>
-    <t>PE 257%PETROLEUM ENGINEERING THERMODYNAMICS I%Sokama-Neuyam Yen Adams%ED2-PE%97%LT/N1/N2/206%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%25/24/24/24</t>
-  </si>
-  <si>
-    <t>CHE 451%CHEMICAL PROCESS DESIGN AND ECONOMICS%Afotey Benjamin%ED4-CHE%114%NAF1/EA/VCR/ECR%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/25/25/24</t>
-  </si>
-  <si>
-    <t>CHE 451%CHEMICAL PROCESS DESIGN AND ECONOMICS%Afotey Benjamin%ED4-PCE%62%N1/N2/RMA%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%22/20/20</t>
-  </si>
-  <si>
-    <t>METE 451%METALLURGICAL PLANT DESIGN/OPERATIONS%Koomson Bennetta%ED4-METE%49%NEB-FF1%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%49</t>
-  </si>
-  <si>
-    <t>IE 455%COSTING AND BREAK-EVEN ANALYSIS%Mensah Lena Dzifa%ED4-IND%67%PB020/PB212%Wednesday, 25 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/27</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Amoako-Yirenkyi Carole Fredua%ED3-ME%230%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%230</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Amoako-Yirenkyi Carole Fredua%ED3-COE%276%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%276</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Amoako-Yirenkyi Carole Fredua%ED3-IND%72%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%72</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%C. F. A. Yirenkyi%ED3-AERO%76%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%76</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Amoako-Yirenkyi Carole Fredua%ED3-GEOM%93%Computer Based%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%93</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Okutu John Kwadey%ED3-EE%254%PB001/PB014/PB020/PB201/PB214/PB208/PB008%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/40/40/40/40/27/27</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%David Benteh%ED3-MARI%40%PB212%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%David Benteh%ED3-GEOL%154%NAF1/EA/A110/VCR/ECR%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25/25</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Okutu John Kwadey%ED3-AUTO%47%VCR/ECR%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%24/24</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%David Benteh%ED3-BME%94%NAF1/EA/A110%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/27/27</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Benteh David%ED3-MSE%89%LT/N2/RMA/RMB%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%25/22/20/20</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Benteh David%ED3-METE%83%VSLA/303/N1%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/25/23</t>
-  </si>
-  <si>
-    <t>STAT 253%PROBABILITY AND STATISTICS%Awiakye-Marfo George%ED3-CE%223%PB014/PB020/PB201/PB214/PB008/PB208%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%42/42/42/42/28/27</t>
-  </si>
-  <si>
-    <t>CE 255%THEORY OF STRUCTURES%Ampofo James Wiafe%ED2-GEOL%154%VSLA/LT/303/RMA/RMB/304%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/25/25/20/20/24</t>
-  </si>
-  <si>
-    <t>CE 255%THEORY OF STRUCTURES%Ampofo James Wiafe%ED2-CE%260%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2/PB001%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%75/75/50/25/35</t>
-  </si>
-  <si>
-    <t>MSE 451%COMPOSITE MATERIALS%Asare Eric Kwame Anokye%ED4-MSE%64%206/N1/N2%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%24/20/20</t>
-  </si>
-  <si>
-    <t>CE 473%DEVELOPMENT ENGINEERING%Tuffour Yaw Adubofour%ED4-CE%245%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 4 (1:30 PM - 2:30 PM)%80/80/55/30</t>
-  </si>
-  <si>
-    <t>CHE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-CHE%120%NAF1/EA/A110/VCR%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30/20</t>
-  </si>
-  <si>
-    <t>CHE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-PCE%56%NEB-FF1%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%56</t>
-  </si>
-  <si>
-    <t>PE 153%ORGANIC CHEMISTRY FOR ENGINEERS%Laryea Michael Konney%ED1-PE%129%VSLA/LT/303/206/N2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/25/20/14</t>
-  </si>
-  <si>
-    <t>MSE 153%INTRODUCTION TO INFORMATION TECHNOLOGY%Okae James%ED1-MSE%98%304/N1/RMA/RMB%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25/24/24</t>
-  </si>
-  <si>
-    <t>MSE 153%INTRODUCTION TO INFORMATION TECHNOLOGY%Okae James%ED1-METE%72%PB201/PB208%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/27</t>
-  </si>
-  <si>
-    <t>METE 251%METALLURGICAL THERMODYNAMICS%Gikunoo Emmanuel%ED2-METE%59%PB214/PB008%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/19</t>
-  </si>
-  <si>
-    <t>TE 353%RANDOM VARIABLES AND STOCHASTIC PROCESSES%Obour Agyekum Kwame Opuni-Boachie%ED3-TEL%147%PB001/PB020/PB014/PB212%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/12</t>
-  </si>
-  <si>
-    <t>ME 355%STRENGTH OF MATERIALS II%Agyei Agyemang Anthony%ED3-AE%105%NEB-SF/NEB-FF2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%80/23</t>
-  </si>
-  <si>
-    <t>AE 471%FARM STRUCTURES%Bart Plange Ato%ED4-AE%103%NAF1/EA/A110%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%43/30/30</t>
-  </si>
-  <si>
-    <t>GE 451%GEODETIC SURVEYING II%Fosu Collins%ED4-GEOM%93%304/N1/RMA/RMB%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/24/22/22</t>
-  </si>
-  <si>
-    <t>EE 167%OCCUPATIONAL HEALTH AND SAFETY%Asiedu Charlotte%ED1-EE%287%PB001/PB020/PB014/PB201/PB214/PB008/PB208/PB212%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/40/40/26/26/20</t>
-  </si>
-  <si>
-    <t>PE 367%STATISTICS FOR PETROLEUM ENGINEERS%Adjei Stephen%ED3-PE%82%NEB-TF%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%82</t>
-  </si>
-  <si>
-    <t>BME 463%BIOMATERIALS II%Agyapong Dorothy Araba Yakoba%ED4-BME%84%NEB-TF%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%84</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Oppong Tawiah Peter%ED1-TEL%129%VSLA/LT/303/206/N2%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/25/20/14</t>
-  </si>
-  <si>
-    <t>GE 263%INFORMATION SCIENCE AND PROGRAMMING%Tienaah Titus%ED2-GEOM%134%NEB-SF/NEB-FF1%Wednesday, 25 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/50</t>
-  </si>
-  <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Andoh Prince Yaw%ED2-ME%242%Computer Based%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%242</t>
-  </si>
-  <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Andoh Prince Yaw%ED2-PE%97%Computer Based%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%97</t>
-  </si>
-  <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Agyei Agyemang Anthony%ED2-AERO%74%NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/24</t>
-  </si>
-  <si>
-    <t>ME 255%STRENGTH OF MATERIALS I%Boahen Samuel%ED2-AE%155%NAF1/EA/A110/ECR/VCR%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/30/30/25/25</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED1-CE%32%PB014%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%32</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED1-GEOL%34%PB020%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%34</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-MSE%13%303%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%13</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-BME%17%PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%17</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTION TO ECONOMICS %Takyi Paul Owusu%ED1-AUTO%88%VSLA/LT/206%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/26/17</t>
-  </si>
-  <si>
-    <t>ECON 151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED2-EE%142%NAF1/EA/A110/ECR/VCR%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/30/30/20/20</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED2-TEL%30%303%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30</t>
-  </si>
-  <si>
-    <t>ECON 151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED2-COE%36%PB001%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%36</t>
-  </si>
-  <si>
-    <t>ECON151%ELEMENTS OF ECONOMICS I%Takyi Paul Owusu%ED3-GEOM%16%PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%16</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED3-PCE%26%PB214%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%26</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTION TO ECONOMICS I%Takyi Paul Owusu%ED3-ME%230%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%85/80/45/20</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTORY ECONOMICS I%Takyi Paul Owusu%ED3-CHE%32%PB201%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/12</t>
-  </si>
-  <si>
-    <t>ECON 151%INTRODUCTION TO ECONOMICS I%Takyi Paul Owusu%ED3-AERO%76%VSLA/LT%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/26</t>
-  </si>
-  <si>
-    <t>TE 455%MICROWAVE ENGINEERING%Abdul-Rahman Ahmed%ED4-TEL%142%NEB-TF/NEB-SF%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/62</t>
-  </si>
-  <si>
-    <t>IE 357%PROJECT MANAGEMENT%Asiedu Charlotte%ED3-IND%72%RMA/RMB/206%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%24/24/24</t>
-  </si>
-  <si>
-    <t>CE 451%STRUCTURAL ENGINEERING I%Osei Jack Banahene%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB208/PB008%Wednesday, 25 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/40/40/40/40/30/15</t>
-  </si>
-  <si>
-    <t>COE 281%PROGRAMMING AND PROBLEM SOLIVING%Adjaidoo Theresa-Samuelle Maame Atwemaah%ED2-COE%253%Computer Based%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%253</t>
-  </si>
-  <si>
-    <t>ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Sackey Michael Nii%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%85/85/52/20</t>
-  </si>
-  <si>
-    <t>ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Asante Eric Amoah%ED2-AE%155%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/30/30/25/25</t>
-  </si>
-  <si>
-    <t>MSE 255%ELECTRICAL AND MAGNETIC BEHAVIOUR OF MATERIALS%Dzikunu Perseverance%ED2-MSE%80%NEB-TF/NEB-FF2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%60/20</t>
-  </si>
-  <si>
-    <t>MSE 255%ELECTRICAL AND MAGNETIC BEHAVIOUR OF MATERIALS%Dzikunu Perseverance%ED2-METE%59%NEB-SF%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%59</t>
-  </si>
-  <si>
-    <t>CE 151%ELEMENTARY STRUCTURES%Afrifa Russel Owusu%ED1-GEOL%119%VSLA/LT/303/RMA%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%50/30/20/20</t>
-  </si>
-  <si>
-    <t>PCE 355%FIRE AND SAFETY ENGINEERING%Momade Zsuzsanna Gál%ED3-PCE%51%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%30/21</t>
-  </si>
-  <si>
-    <t>CHE 459%SAFETY AND POLLUTION CONTROL%Ohemeng-Boahen Godfred%ED4-CHE%114%VSLA/LT/303/RMA%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%44/30/20/20</t>
-  </si>
-  <si>
-    <t>GED 267%COMPUTER PROGRAMMING%Kwaw Albert Kwame%ED2-GEOL%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/30/30/25/25</t>
-  </si>
-  <si>
-    <t>EE 387%CLASSICAL CONTROL SYSTEMS%Opoku Daniel%ED3-EE%254%PB001/PB020/PB014/PB201/PB214/PB008%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/45/45/45/45/30</t>
-  </si>
-  <si>
-    <t>MME 353%MARINE ELECTRICAL TECHNOLOGY%Frimpong Emmanuel Asuming%ED3-MARI%40%PB008/PB208%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20</t>
-  </si>
-  <si>
-    <t>GE 171%APPLIED OPTICS%Andam-Akorful Samuel Ato%ED1-GEOM%100%304/N1/RMB/206/N2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%25/25/20/20/10</t>
-  </si>
-  <si>
-    <t>COE 387%CLASSICAL CONTROL SYSTEMS%Klogo Griffith Selorm%ED3-BME%94%304/N1/RMB/206/N2%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%20/20/20/20/10</t>
-  </si>
-  <si>
-    <t>COE 387%CLASSICAL CONTROL SYSTEMS%Klogo Griffith Selorm%ED3-COE%276%PB001/PB020/PB014/PB201/PB214/PB208/PB212%Thursday, 26 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/45/45/45/45/30/21</t>
-  </si>
-  <si>
-    <t>CHE 261%COMPUTER APPLICATIONS FOR ENGINEERS%Bonsu Jude Kwaku%ED2-PCE%59%Computer Based%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%59</t>
-  </si>
-  <si>
-    <t>CHE 261%COMPUTER APPLICATIONS FOR ENGINEERS%Anang Daniel Adjah%ED2-CHE%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/30/30/25/25</t>
-  </si>
-  <si>
-    <t>CE 151%ELEMENTARY STRUCTURES%Afrifa Russel Owusu%ED1-CE%242%PB001/PB020/PB014/PB201/PB214/PB208%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/45/45/20</t>
-  </si>
-  <si>
-    <t>MSE 155%PRINCIPLES OF MATERIALS SCIENCE%Nartey Martinson Addo%ED1-MSE%98%PB208/PB008/PB214%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/30/38</t>
-  </si>
-  <si>
-    <t>ME 365%THERMODYNAMICS  II%Forson Francis Kofi%ED3-AE%105%NAF1/EA/A110/ECR%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%40/25/20/20</t>
-  </si>
-  <si>
-    <t>ME 365%THERMODYNAMICS  II%Forson Francis Kofi%ED3-ME%230%PB001/PB020/PB014/PB201/PB008/PB212%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/42/43/30/25</t>
-  </si>
-  <si>
-    <t>CE 463%WATER AND WASTE WATER ENGINEERING%Buamah Richard Akwasi%ED4-CE%245%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%85/85/52/23</t>
-  </si>
-  <si>
-    <t>COE 281%PROGRAMMING AND PROBLEM SOLIVING%Adjei Prince Ebenezer%ED2-BME%87%VSLA/LT/RMA%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/21/21</t>
-  </si>
-  <si>
-    <t>TE 251%ANALOG COMMUNICATION SYSTEMS%Affum Emmanuel Ampoma%ED2-TEL%179%VSLA/RMA/303/304/N1/N2/206%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/20/30/22/25/20/17</t>
-  </si>
-  <si>
-    <t>METE 351%PRINCIPLES OF HYDROMETALLURGY%Koomson Bennetta%ED3-METE%83%303/LT/RMB%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/30/23</t>
-  </si>
-  <si>
-    <t>MSE 355%POLYMER PROCESSING%Asare Eric Kwame Anokye%ED3-MSE%89%304/N1/RMB/206%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%25/25/20/20</t>
-  </si>
-  <si>
-    <t>CHE 455%PROCESS CONTROL AND INSTRUMENTATION%Baidoo Martina Francisca%ED4-PCE%62%NEB-TF%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%62</t>
-  </si>
-  <si>
-    <t>PE 357%PETROLEUM PRODUCTION ENGINEERING I%Sarkodie Kwame%ED3-PE%82%NEB-SF%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%82</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Ayetor Godwin Kafui Kwesi%ED2-MARI%37%Computer Based %Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%Computer Based </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Ayetor Godwin Kafui Kwesi%ED2-AUTO%77%Computer Based %Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%Computer Based </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME 259%APPLICATIONS OF COMPUTER GRAPHICS%Ayetor Godwin Kafui Kwesi%ED2-IND%80%Computer Based %Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%Computer Based </t>
-  </si>
-  <si>
-    <t>AERO 351%AERODYNAMICS I%Bofah Kwasi Kete%ED3-AERO%76%304/N1/N2/RMA%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%20/20/20/16</t>
-  </si>
-  <si>
-    <t>GED 369%PHOTOGEOLOGY AND REMOTE SENSING%Nuamah Daniel Oduro Boatey%ED3-GEOL%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/30/30/25/25</t>
-  </si>
-  <si>
-    <t>GE 361%IMAGE PROCESSING AND INTERPRETATION%Asare Yaw Mensah %ED3-GEOM%115%NEB-SF/NEB-FF1%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%70/45</t>
-  </si>
-  <si>
-    <t>GED 461%EXPLORATION GEOPHYSICS%Ali Bukari%ED4-GEOL%102%VSLA/LT/303%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%50/26/26</t>
-  </si>
-  <si>
-    <t>CE 259%ENGINEERING GEOLOGY%Acquaah Vincent Kofi Abaka%ED2-CE%260%PB001/PB020/PB014/PB201/PB214/PB208/PB212%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/45/45/40/20/20</t>
-  </si>
-  <si>
-    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Mensah Lena Dzifa%ED4-ME%144%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/30/30/25/15</t>
-  </si>
-  <si>
-    <t>ME 491%ENGINEERING ECONOMICS AND MANAGEMENT%Mensah Lena Dzifa%ED4-EE%224%PB001/PB020/PB014/PB201/PB214%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/45/45/44</t>
-  </si>
-  <si>
-    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Mensah Lena Dzifa%ED4-IND%67%NEB-TF%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%67</t>
-  </si>
-  <si>
-    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Mensah Lena Dzifa%ED4-MSE%64%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40/24</t>
-  </si>
-  <si>
-    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Mensah Lena Dzifa%ED4-METE%49%RMB/206%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%24/25</t>
-  </si>
-  <si>
-    <t>MME 491%MARINE ENGINEERING ECONOMY, ACCOUNTING AND MANAGEMENT%Mensah Lena Dzifa%ED4-MARI%23%RMB%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%23</t>
-  </si>
-  <si>
-    <t>AERO 491%AVIATION BUSINESS MANAGEMENT%Takyi Gabriel%ED4-AERO%61%PB008/PB208/PB212%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%20/25/16</t>
-  </si>
-  <si>
-    <t>ME 491%ENGINEERING ECONOMY AND MANAGEMENT%Asiedu Charlotte%ED4-AUTO%32%PB008%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%32</t>
-  </si>
-  <si>
-    <t>ME 491%ENGINEERING ECONOMICS AND MANAGEMENT%Mensah Lena Dzifa%ED4-COE%170%NEB-TF/NEB-SF%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%85/85</t>
-  </si>
-  <si>
-    <t>ME 491%ENGINEERING ECONOMICS AND MANAGEMENT%Aikins Stephen Hill Mends%ED4-AE%103%VSLA/LT/303%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%50/26/27</t>
-  </si>
-  <si>
-    <t>ME 491%ENGINEERING ECONOMICS AND MANAGEMENT%Mensah Lena Dzifa%ED4-BME%84%304/N1/N2/RMA%Thursday, 26 February 2026%Session, 3 (11:45 AM - 12:45 PM)%25/25/20/14</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Abdul-Rahman Ahmed%ED1-TEL%129%NAF1/EA/A110/VCR%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Acheampong Francisca Adoma%ED1-AUTO%88%N1/N2/206/304%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%22/22/22/22</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Acheampong Francisca Adoma%ED1-MARI%46%N2/RMA%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%23/23</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Affum Emmanuel Ampoma%ED1-ME%223%NEB-TF/NEB-SF/NEB-FF1%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%85/85/55</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Evils Twumasi%ED1-METE%72%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/22</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Ellis Sani Mubarak%ED1-PE%129%NAF1/EA/A110/ECR%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Evils Twumasi%ED1-CHE%120%NEB-SF/NEB-FF2%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%85/35</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Prah II Nicholas Kwesi%ED1-AE%126%VSLA/LT/RMA/RMB%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/30/24/24</t>
-  </si>
-  <si>
-    <t>COE 181%APPLIED ELECTRICITY%Oteng Gyasi Kwame%ED1-COE%261%PB001/PB020/PB014/PB201/PB214/PB008/PB212%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/45/45/45/45/30/6</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Effah Francis Boafo%ED1-EE%287%PB001/PB020/PB014/PB201/PB214/PB008/PB208/PB212%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/45/45/45/45/30/30/2</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Evils Twumasi%ED1-PCE%56%ECR/VCR%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/26</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Obeng Kwakye Kingsford Sarkodie%ED1-IND%81%NEB-TF%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%81</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Oteng Gyasi Kwame%ED1-AERO%70%PB208/PB212%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/40</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Obeng Kwakye Kingsford Sarkodie%ED1-BME%136%VSLA/LT/303/N1%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%50/30/30/26</t>
-  </si>
-  <si>
-    <t>EE 151%APPLIED ELECTRICITY%Oteng Gyasi Kwame%ED1-MSE%98%303/304/RMB/206%Thursday, 26 February 2026%Session, 4 (1:30 PM - 2:30 PM)%30/25/24/24</t>
-  </si>
-  <si>
-    <t>COE 475%COMPUTER NETWORKING%Akowuah Emmanuel Kofi%ED4-COE%170%Computer Based%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%170</t>
-  </si>
-  <si>
-    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-AERO%74%PB201/PB208/PB212%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/14</t>
-  </si>
-  <si>
-    <t>ME 261%ENGINEERING MECHANICS II: DYNAMICS%Ampofo Joshua%ED2-ME%242%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/80/50/27</t>
-  </si>
-  <si>
-    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-MARI%37%A110/ECR%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/17</t>
-  </si>
-  <si>
-    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-IND%80%VSLA/LT%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%50/30</t>
-  </si>
-  <si>
-    <t>ME 261%ENGINEERING MECHANICS II:DYNAMICS%Ampofo Joshua%ED2-AUTO%77%N1/RMA/206/N2%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20/20/17</t>
-  </si>
-  <si>
-    <t>MSE 361%STRESS AND STRAIN ANALYSIS OF RIGID BODIES%Mensah-Darkwa Kwadwo%ED3-MSE%89%NAF1/EA/VCR%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/30/14</t>
-  </si>
-  <si>
-    <t>METE 353%STRENGTH OF MATERIALS%Mensah-Darkwa Kwadwo%ED3-METE%83%303/304/RMA/RMB%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%30/20/20/13</t>
-  </si>
-  <si>
-    <t>IE 367%ETHICS, CONTRACT &amp; PRODUCT LIABILITY LAW%Asiedu Charlotte%ED3-IND%72%PB214/PB008%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%42/30</t>
-  </si>
-  <si>
-    <t>MSE 257%MATERIALS PROCESSING%Agyemang Frank Ofori%ED2-MSE%80%NAF1/EA/VCR%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/20/15</t>
-  </si>
-  <si>
-    <t>PCE 457%CORROSION ENGINEERING%Anang Daniel Adjah%ED4-PCE%62%RMB/206/N1%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20/22</t>
-  </si>
-  <si>
-    <t>AE 351%SOIL AND WATER ENGINEERING%Kyei-Baffour Nicholas%ED3-AE%105%VSLA/LT/303%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%50/28/27</t>
-  </si>
-  <si>
-    <t>TE 271%ANALOG COMMUNICATION SYSTEMS%Ellis Sani Mubarak%ED3-EE%254%NEB-TF/NEB-SF/NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/85/55/29</t>
-  </si>
-  <si>
-    <t>CHE 371%NATURAL GAS PROCESSING TECHNOLOGY%Benjamin Asante%ED3-CHE%50%PB208/PB008%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25</t>
-  </si>
-  <si>
-    <t>TE 453%MOBILE AND WIRELESS COMMUNICATIONS%Agyekum Kwame Agyeman-Prempeh%ED4-TEL%142%PB001/PB020/PB014/PB212%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/40/42/15</t>
-  </si>
-  <si>
-    <t>ME 361%DYNAMICS OF MACHINERY%Ampofo Joshua%ED3-MARI%40%N2/206%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%20/20</t>
-  </si>
-  <si>
-    <t>ME 361%DYNAMICS OF MACHINERY%Ampofo Joshua%ED3-AUTO%47%A110/ECR%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/22</t>
-  </si>
-  <si>
-    <t>ME 361%DYNAMICS OF MACHINERY%Sackey Samuel Mensah%ED3-ME%230%PB001/PB020/PB014/PB201/PB214/PB212%Thursday, 26 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/40/40/40/20</t>
-  </si>
-  <si>
-    <t>GE 371%SURVEY ADJUSTMENT I%Fosu Collins%ED3-GEOM%115%Computer Based%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%115</t>
-  </si>
-  <si>
-    <t>GE 271%ENGINEERING SURVEYING I%Arko-Adjei Anthony%ED2-GEOM%134%PB214/PB212/PB208/PB008%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/29/30/30</t>
-  </si>
-  <si>
-    <t>CHE 251%CHEMICAL PROCESS CALCULATIONS I%Rockson Mizpah Ama Dziedzorm%ED2-CHE%154%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/30/30/25/25</t>
-  </si>
-  <si>
-    <t>CHE 251%CHEMICAL PROCESS CALCULATIONS I%Ohemeng-Boahen Godfred%ED2-PCE%59%PB208/PB008%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%30/29</t>
-  </si>
-  <si>
-    <t>ARC 155%CLIMATE AND ARCHITECTURE%Amos-Abanyie Samuel%ED1-CE%74%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/24</t>
-  </si>
-  <si>
-    <t>PE 359%RESERVOIR PETROPHYSICS%Erzuah Samuel%ED3-PE%82%NEB-SF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%82</t>
-  </si>
-  <si>
-    <t>CE 479%ENGINEERING AND ENVIRONMENTAL GEOPHYSICS%Owusu-Nimo Frederick%ED4-CE%245%VSLA/LT/RMA/RMB/303/304/206/N1/N2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%50/25/24/24/30/21/24/25/22</t>
-  </si>
-  <si>
-    <t>PE 451%PETROLEUM ECONOMICS%Quaye Jonathan Atuquaye%ED4-PE%103%NEB-SF/NEB-FF2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/23</t>
-  </si>
-  <si>
-    <t>PE 255%FLUID MECHANICS%Adjei Stephen%ED2-PE%97%NEB-TF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%97</t>
-  </si>
-  <si>
-    <t>TE 253%DIGITAL SYSTEMS%Obour Agyekum Kwame Opuni-Boachie%ED2-TEL%179%PB001/PB020/PB014/PB201%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45</t>
-  </si>
-  <si>
-    <t>TE 355%SIGNALS AND SYSTEMS%Agyekum Kwame Agyeman-Prempeh%ED3-TEL%147%NAF1/EA/A110/ECR/VCR%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/30/30/21/21</t>
-  </si>
-  <si>
-    <t>PCE 357%ORGANIC AND PETROCHEMICAL SYNTHESIS%Mensah Mary%ED3-PCE%51%NEB-TF%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%51</t>
-  </si>
-  <si>
-    <t>CE 353%REINFORCED CONCRETE DESIGN%Owusu Twumasi Jones%ED3-CE%223%PB001/PB020/PB014/PB201/PB214/PB212%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%41/42/40/40/40/20</t>
-  </si>
-  <si>
-    <t>GE 161%BASIC SURVEY PRINCIPLES I%Ayer John Wise Divine%ED1-GEOM%100%VSLA/LT/RMA/RMB%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/20/20/20</t>
-  </si>
-  <si>
-    <t>GE 475%RESEARCH METHODS%Duker Alfred Alan%ED4-GEOM%93%303/304/206/N1/N2%Thursday, 26 February 2026%Session, 6 (5:00 PM - 6:00 PM)%25/18/18/18/14</t>
-  </si>
-  <si>
-    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sackey Michael Nii%ED1-AERO%70%NAF1/A110%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%42/28</t>
-  </si>
-  <si>
-    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sackey Michael Nii%ED1-ME%223%VSLA/LT/303/304/N1/RMA/RMB/206/N2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%44/26/26/22/22/21/21/21/20</t>
-  </si>
-  <si>
-    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sekyere Charles Kofi Kafui%ED1-MARI%46%A110/VCR%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%23/23</t>
-  </si>
-  <si>
-    <t>ME 157%INTRODUCTION TO INFORMATION TECHNOLOGY%Sekyere Charles Kofi Kafui%ED1-IND%81%303/304/206/RMB%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%25/20/20/20</t>
-  </si>
-  <si>
-    <t>EE 271%SEMICONDUCTOR DEVICES%Sekyere Yaw Opoku Mensah%ED2-EE%340%PB001/PB014/PB020/PB201/PB214/PB008/PB208/PB212/EA%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%45/45/45/45/45/30/30/25/30</t>
-  </si>
-  <si>
-    <t>COE 271%SEMICONDUCTOR DEVICES%Kommey Benjamin%ED2-BME%87%VSLA/LT/RMA%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%40/27/21</t>
-  </si>
-  <si>
-    <t>COE 271%SEMICONDUCTOR DEVICES%Kommey Benjamin%ED2-COE%253%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%85/85/55/28</t>
-  </si>
-  <si>
-    <t>EE 371%LINEAR ELECTRONIC CIRCUITS%Sekyere Yaw Opoku Mensah%ED3-EE%254%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%85/85/55/29</t>
-  </si>
-  <si>
-    <t>IE 365%ENGINEERING WORK STUDY%Takyi Gabriel%ED3-IND%72%NAF1/EA%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%44/28</t>
-  </si>
-  <si>
-    <t>EE 153%ELECTRICAL ENGINEERING TECHNOLOGY WITH MATLAB%Prah II Nicholas Kwesi%ED1-EE%287%PB001/PB014/PB020/PB201/PB214/PB208/PB008/PB212%Friday, 27 February 2026%Session, 1 (8:15 AM - 9:15 AM)%42/42/42/42/42/30/28/20</t>
-  </si>
-  <si>
-    <t>GED 151%BASIC GEOLOGY%Gawu Simon Kafui Yawo%ED1-GEOL%119%VSLA/RMA/303/N2%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/30/24/15</t>
-  </si>
-  <si>
-    <t>PE 253%BASIC GEOLOGY%Quaye Jonathan Atuquaye%ED2-PE%97%LT/304/RMA/206%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/25/24/18</t>
-  </si>
-  <si>
-    <t>AE 373%MACHINE DESIGN I%Aveyire Joseph%ED3-AE%105%VSLA/304/RMB/N2%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/25/24/6</t>
-  </si>
-  <si>
-    <t>PE 155%INTRODUCTION TO INFORMATION TECHNOLOGY%Sokama-Neuyam Yen Adams%ED1-PE%129%PB020/PB201/PB008/PB212%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/30/9</t>
-  </si>
-  <si>
-    <t>CHE 253%CHEMICAL ENGINEERING THERMODYNAMICS I%Bonsu Jude Kwaku%ED2-CHE%154%PB001/PB014/PB214/PB208%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/19</t>
-  </si>
-  <si>
-    <t>CHE 253%CHEMICAL ENGINEERING THERMODYNAMICS I%Dogbe Eunice Sefakor Aku%ED2-PCE%59%NAF1/A110%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%39/20</t>
-  </si>
-  <si>
-    <t>AERO 391%AEROSPACE INDUSTRY AND ENGINEERING%K. K. Bofah%ED3-AERO%76%NEB-TF%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/25/21</t>
-  </si>
-  <si>
-    <t>MSE 253%MECHANICAL BEHAVIOUR OF MATERIALS%Kwofie Samuel%ED2-MSE%80%LT/N1/RMB%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%30/25/25</t>
-  </si>
-  <si>
-    <t>MSE 253%MECHANICAL BEHAVIOUR OF MATERIALS%Kwofie Samuel%ED2-METE%59%303/N1/206%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%20/20/19</t>
-  </si>
-  <si>
-    <t>GE 251%PRINCIPLES OF PHOTOGRAMMETRY%Ahorsu Harriet Atsufui%ED2-GEOM%134%PB020/PB201/PB008/PB212%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/30/14</t>
-  </si>
-  <si>
-    <t>CE 153%ENGINEERING PRACTICE AND TECHNOLOGY%Acquaah Vincent Kofi Abaka%ED1-CE%242%NEB-SF/NEB-FF1/NEB-FF2/NAF1/EA/VCR%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%80/50/20/40/30/25</t>
-  </si>
-  <si>
-    <t>CE 251%STRENGTH OF MATERIALS%Amponsah Evans%ED2-CE%260%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%85/85/55/35</t>
-  </si>
-  <si>
-    <t>CE 251%STRENGTH OF MATERIALS%Kankam Charles Kwame%ED2-GEOL%154%PB001/PB014/PB214/PB208%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%45/45/45/19</t>
-  </si>
-  <si>
-    <t>CHE 363%POLYMER TECHNOLOGY%Boakye Patrick%ED3-CHE%36%ECR/VCR%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%25/11</t>
-  </si>
-  <si>
-    <t>CHE 363%POLYMER TECHNOLOGY%Boakye Patrick%ED3-PCE%51%A110/EA%Friday, 27 February 2026%Session, 2 (10:00 AM - 11:00 AM)%31/20</t>
-  </si>
-  <si>
-    <t>EE 287%CIRCUIT THEORY%Gadze James Dzisi%ED2-TEL%179%PB001/PB014/PB214/PB208/PB212%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/45/38/9</t>
-  </si>
-  <si>
-    <t>COE 475%COMPUTER NETWORKING%Adrah Charles Mawutor%ED4-EE%224%PB001/PB020/PB014/PB201/PB008/PB212%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/45/45/30/14</t>
-  </si>
-  <si>
-    <t>TE 465%DIGITAL INTEGRATED CIRCUITS%Affum Emmanuel Ampoma%ED4-TEL%142%PB020/PB201/PB008/PB208%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/45/30/22</t>
-  </si>
-  <si>
-    <t>IE 457%ADVANCED MANUFACTURING TECHNOLOGY II%Takyi Gabriel%ED4-IND%67%PB214/PB212%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/22</t>
-  </si>
-  <si>
-    <t>GE 381%ENGINEERING SURVEYING I%Obeng Kwame%ED3-CE%223%NEB-SF/NEB-TF/NEB-FF1%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%85/85/53</t>
-  </si>
-  <si>
-    <t>MSE 457%METALWORKING PROCESSES%Kwofie Samuel%ED4-MSE%64%304/RMA/N2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%25/24/15</t>
-  </si>
-  <si>
-    <t>MSE 457%METAL FORMING PROCESSES%Kwofie Samuel%ED4-METE%49%A110/ECR%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%30/19</t>
-  </si>
-  <si>
-    <t>CHE 463%ELECTROCHEMICAL TECHNOLOGY%Anang Daniel Adjah%ED4-PCE%18%A110%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%18</t>
-  </si>
-  <si>
-    <t>CHE 463%ELECTROCHEMICAL TECHNOLOGY%Anang Daniel Adjah%ED4-CHE%40%NAF1%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%40</t>
-  </si>
-  <si>
-    <t>CE 477%GEOTECHNICAL ENGINEERING I%Ayeh Felix Jojo Fianko%ED4-CE%245%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%80/80/55/30</t>
-  </si>
-  <si>
-    <t>CE 477%GEOTECHNICAL ENGINEERING I%Ampadu Samuel Innocent Kofi%ED4-GEOL%102%LT/303/RMA/206%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%30/30/24/18</t>
-  </si>
-  <si>
-    <t>AE 451%IRRIGATION AND DRAINAGE%Agodzo Sampson Kwaku%ED4-AE%103%VSLA/N1/RMB/N2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%45/25/24/9</t>
-  </si>
-  <si>
-    <t>PE 361%RESERVOIR ENGINEERING II%Adenutsi Caspar Daniel%ED3-PE%82%303/N1/206%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%30/25/27</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Amoabeng Kofi Owura%ED1-BME%136%VSLA/LT/304/RMB/N2%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%50/30/25/24/7</t>
-  </si>
-  <si>
-    <t>MME 473%MARINE MACHINERY SYSTEM DESIGN%Sackey Michael Nii%ED4-MARI%23%ECR%Friday, 27 February 2026%Session, 3 (11:45 AM - 12:45 PM)%23</t>
-  </si>
-  <si>
-    <t>COE 253%DISCRETE STRUCTURES%Kwabi Prince Amponsah%ED2-COE%253%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%85/85/53/30</t>
-  </si>
-  <si>
-    <t>ME 451%BEHAVIOUR OF REAL FLUIDS%Opoku Richard%ED4-ME%144%NAF1/EA/A110/VCR/ECR%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40/30/30/25/20</t>
-  </si>
-  <si>
-    <t>ME 451%BEHAVIOUR OF REAL FLUIDS%Opoku Richard%ED4-AERO%61%RMA/RMB/206%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%21/20/20</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-MSE%98%PB201/PB208/PB212%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%43/30/25</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-TEL%129%PB001/PB014/PB020%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%43/43/43</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-MARI%46%N2/206%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%23/23</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Sunnu Albert Kojo%ED1-ME%223%VSLA/LT/303/304/RMA/RMB/N1/N2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/24/24/24/24/23</t>
-  </si>
-  <si>
-    <t>SES 171%FUNDAMENTALS OF ACQUATIC SKILLS%Afrifa Daniel%ED2-MARI%40%PB214%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%40</t>
-  </si>
-  <si>
-    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-ME%242%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%81/81/50/30</t>
-  </si>
-  <si>
-    <t>ME 251%INTRODUCTION TO FLUID MECHANICS%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-AERO%74%NAF1/A110%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%44/30</t>
-  </si>
-  <si>
-    <t>ME 251%FLUID MECHANICS I%Fiagbe Yesuenyeagbe Atsu Kwabla%ED2-AE%155%VSLA/LT/303/N1/304%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/30/30/25/24</t>
-  </si>
-  <si>
-    <t>AME 371%LAND VEHICLE DESIGN%Ayetor Godwin Kafui Kwesi%ED3-AUTO%47%VCR/ECR%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%24/23</t>
-  </si>
-  <si>
-    <t>EE 261%DC MACHINES%Effah Francis Boafo%ED2-EE%340%PB001/PB014/PB020/PB201/PB214/PB008/PB208/PB212/EA%Friday, 27 February 2026%Session, 4 (1:30 PM - 2:30 PM)%45/45/45/45/45/30/30/25/30</t>
-  </si>
-  <si>
-    <t>IE 363%PROCESS PLANNING SYSTEMS%Sackey Samuel Mensah%ED3-IND%72%ECR/VCR/A110%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%25/25/22</t>
-  </si>
-  <si>
-    <t>MSE 363%MATERIALS CHARACTERIZATION TECHNIQUE%Arthur Emmanuel Kwesi%ED3-METE%83%RMA/RMB/N1/206%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%21/21/21/20</t>
-  </si>
-  <si>
-    <t>MSE 363%MATERIALS CHARACTERIZATION TECHNIQUE%Arthur Emmanuel Kwesi%ED3-MSE%89%NEB-TF/NEB-FF2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%64/25</t>
-  </si>
-  <si>
-    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-COE%276%PB001/PB020/PB014/PB201/PB214/PB008/PB212%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/45/45/30/21</t>
-  </si>
-  <si>
-    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-BME%94%NAF1/EA/VCR%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/24</t>
-  </si>
-  <si>
-    <t>COE 381%MICROPROCESSORS%Keelson Eliel%ED3-EE%254%PB001/PB020/PB014/PB201/PB214/PB208%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/45/45/45/45/29</t>
-  </si>
-  <si>
-    <t>CHE 351%MASS TRANSFER PROCESSES%Ankudey Emmanuel Godwin%ED3-CHE%100%NAF1/EA/A110%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Boahen Samuel%ED1-GEOL%119%VSLA/LT/303/304%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%45/25/25/24</t>
-  </si>
-  <si>
-    <t>BME 265%BIOLOGICAL TRANSPORT PHENOMENA%Odame Prince%ED2-BME%87%RMA/RMB/N1/N2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%22/22/22/21</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Boahen Samuel%ED1-PCE%56%PB208/PB008%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%28/28</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Asante Eric Amoah%ED1-CHE%120%VSLA/LT/303/304%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%40/30/30/20</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Aveyire Joseph%ED1-CE%242%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%85/85/50/22</t>
-  </si>
-  <si>
-    <t>ME 159%TECHNICAL DRAWING%Aveyire Joseph%ED1-AE%126%NEB-SF/NEB-FF1%Friday, 27 February 2026%Session, 5 (3:15 PM - 4:15 PM)%75/51</t>
-  </si>
-  <si>
-    <t>CE 359%SOIL MECHANICS%Charkley Frederick Nai%ED3-CE%223%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%75/75/50/23</t>
-  </si>
-  <si>
-    <t>GED 379%SOIL MECHANICS%Amenuvor Andrew Cudzo%ED3-GEOL%154%VSLA/LT/303/304/206%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%49/30/30/25/20</t>
-  </si>
-  <si>
-    <t>PE 259%SURVIVAL SWIMMING TECHNIQUES%Gyamfi Isaac%ED2-PE%97%VSLA/LT/303/304/206%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/25/20/12</t>
-  </si>
-  <si>
-    <t>PCE 451%CATALYSIS%Baidoo Martina Francisca%ED4-PCE%62%N1/RMA/RMB%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%22/20/20</t>
-  </si>
-  <si>
-    <t>ME 373%MACHINE ELEMENTS DESIGN I%Davis Francis%ED3-ME%230%NEB-SF/NEB-TF/NEB-FF1/NEB-FF2%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%80/80/50/20</t>
-  </si>
-  <si>
-    <t>GE 351%STEREO PHOTOGRAMMETRY%Tienaah Titus%ED3-GEOM%115%NAF1/EA/A110/VCR%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/30/30/15</t>
-  </si>
-  <si>
-    <t>ME 161%BASIC MECHANICS%Tay Godwin Fabiola Kwaku%ED1-COE%261%PB001/PB020/PB014/PB201/PB214/PB208/PB212%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%42/42/42/42/42/30/21</t>
-  </si>
-  <si>
-    <t>MME 365%ENGINEERING THERMODYNAMICS%Amoabeng Kofi Owura%ED3-MARI%40%ECR/VCR%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%20/20</t>
-  </si>
-  <si>
-    <t>AME 485%AUTOMATIC POWER TRAIN%Abu Frimpong Solomon%ED4-AUTO%32%RMA/RMB%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%16/16</t>
-  </si>
-  <si>
-    <t>CE 461%ENG ECONOMY AND ENTERPRENEURSHIP DEVELOPMENT%Appiah-Effah Eugene%ED4-GEOM%93%NAF1/EA/A110%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%40/25/28</t>
-  </si>
-  <si>
-    <t>CE 461%ENGINEERING ECONOMY AND ENTERPRENEURSHIP%Appiah-Effah Eugene%ED4-CE%245%PB001/PB020/PB014/PB201/PB214/PB212%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%45/45/45/45/45/20</t>
-  </si>
-  <si>
-    <t>ME 455%FINITE ELEMENT METHODS%Andoh Prince Yaw%ED4-ME%144%Computer Based%Friday, 27 February 2026%Session, 6 (5:00 PM - 6:00 PM)%144</t>
-  </si>
-  <si>
-    <t>GE 151%CARTOGRAPHY I%Quaye-Ballard Jonathan Arthur%ED1-GEOM%100%PB008/PB208/PB214/PB212%Monday, 23 February 2026%Session, 1 (8:15AM - 9:15 AM)%30/30/20/20</t>
-  </si>
-  <si>
-    <t>GED 253%PHYSICAL GEOLOGY%Mensah Emmanuel%ED2-GEOL%154%PB014/PB001/PB020/PB008%Monday, 23 February 2026%Session, 1 (8:15AM - 9:15 AM)%40/44/40/30</t>
-  </si>
-  <si>
-    <t>CHE 255%FLUID TRANSPORT%Dogbe Eunice Sefakor Aku%ED2-PCE%59%PB214/PB201%Monday, 23 February 2026%Session, 2  (10:00AM - 11:00 AM)%30/29</t>
-  </si>
-  <si>
-    <t>GED 251%MINERALOGY%Wilson Matthew Coffie%ED2-GEOL%154%NEB-SF/NEB-FF1/NEB-FF2%Monday, 23 February 2026%Session, 5 (3:15PM - 4:15 PM)%80/50/24</t>
   </si>
   <si>
     <t>MSE 155%PRINCIPLES OF MATERIALS SCIENCE%Nartey Martinson Addo%ED1-METE%72%NEB-FF1/NEB-FF2%Thursday, 26 February 2026%Session, 2 (10:00 AM - 11:00 AM)%50/22</t>
@@ -1831,7 +1822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A480"/>
+  <dimension ref="A1:A477"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="212.36328125" bestFit="1" customWidth="1"/>
@@ -1949,7 +1940,7 @@
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
@@ -1974,7 +1965,7 @@
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
@@ -1994,7 +1985,7 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
@@ -2299,22 +2290,22 @@
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>89</v>
+        <v>474</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>478</v>
+        <v>91</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.35">
@@ -2574,1667 +2565,1652 @@
     </row>
     <row r="148" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>143</v>
+        <v>475</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="150" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="151" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="158" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="159" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="160" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="161" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="162" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="163" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="173" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="174" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="175" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="176" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="179" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="180" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="181" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="182" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="185" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="187" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="188" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="189" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="190" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="191" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="192" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="199" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="200" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="201" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="202" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="203" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="204" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="205" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="206" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="209" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="210" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="211" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="212" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="213" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="214" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="215" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="216" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="217" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="218" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="219" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="220" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="221" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="222" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="223" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="224" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="225" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="226" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="227" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="228" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="229" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="230" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="233" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="235" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="236" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="237" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="238" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="239" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="240" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="241" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="242" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="245" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="246" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="247" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="248" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="249" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="250" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="251" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="252" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="253" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="254" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="256" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="257" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="258" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="259" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="260" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="261" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="262" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="263" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="264" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="265" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="266" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="267" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="268" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="269" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="270" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="271" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="272" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="273" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="274" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="275" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="276" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="277" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="278" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="279" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="280" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="281" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="282" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="283" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="284" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="285" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="286" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="287" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="288" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="289" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="290" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="291" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="292" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="293" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="294" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="295" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="296" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="297" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="298" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="299" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="300" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="301" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="302" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="303" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="304" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="305" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="306" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="307" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="308" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="309" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="310" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="311" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="312" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="313" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="314" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="315" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="316" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="317" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="318" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="319" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="320" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="321" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="322" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
-        <v>317</v>
+        <v>476</v>
       </c>
     </row>
     <row r="323" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="324" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="325" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
-        <v>479</v>
+        <v>318</v>
       </c>
     </row>
     <row r="326" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="327" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="328" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="329" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="330" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="331" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="332" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="333" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="334" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="335" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="336" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="337" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="338" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="339" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="340" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="341" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="342" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="343" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="344" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="345" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A345" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="346" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="347" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A347" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="348" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="349" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A349" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="350" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A350" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="351" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="352" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="353" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A353" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="354" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A354" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="355" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A355" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="356" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A356" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="357" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="358" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="359" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="360" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="361" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="362" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="363" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="364" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="365" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="366" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="367" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="368" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="369" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="370" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A370" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="371" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A371" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="372" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A372" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="373" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A373" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="374" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A374" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="375" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A375" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="376" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A376" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="377" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A377" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="378" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="379" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="380" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="381" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="382" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="383" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A383" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="384" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="385" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A385" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="386" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A386" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="387" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A387" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="388" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A388" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="389" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A389" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="390" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A390" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="391" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A391" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="392" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A392" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="393" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A393" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="394" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="395" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="396" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A396" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="397" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A397" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="398" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A398" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="399" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A399" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="400" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="401" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="402" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="403" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A403" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="404" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A404" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="405" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="406" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="407" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A407" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="408" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A408" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="409" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A409" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="410" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="411" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A411" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="412" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A412" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="413" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A413" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="414" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="415" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="416" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A416" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="417" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A417" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="418" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A418" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="419" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A419" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="420" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A420" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="421" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A421" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="422" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A422" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="423" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A423" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="424" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A424" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="425" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A425" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="426" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A426" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="427" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A427" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="428" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A428" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="429" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A429" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="430" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A430" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="431" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A431" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="432" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A432" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="433" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A433" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="434" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="435" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="436" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A436" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="437" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="438" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A438" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="439" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A439" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="440" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A440" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="441" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A441" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="442" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="443" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A443" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="444" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A444" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="445" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A445" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="446" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A446" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="447" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A447" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="448" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A448" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="449" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A449" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="450" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A450" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="451" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A451" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="452" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A452" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="453" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A453" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="454" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="455" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="456" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A456" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="457" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A457" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="458" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A458" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="459" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A459" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="460" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A460" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="461" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A461" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="462" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A462" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="463" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A463" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="464" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A464" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="465" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A465" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="466" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A466" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="467" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A467" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="468" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A468" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="469" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A469" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="470" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A470" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="471" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A471" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="472" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A472" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="473" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A473" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="474" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A474" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="475" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A475" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="476" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A476" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="477" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A477" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="478" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A478" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="479" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A479" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="480" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A480" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>

</xml_diff>